<commit_message>
Render bundled demo verisini gerçekçi lokal veriyle güncelle
Bundled demo-data/current klasörü hala eski (16 Eylül, gerçekçilik
dönüşümünden önceki) sentetik verileri içeriyordu; bu yüzden Render'da
isim/soyisim, seri no ve hostname'ler localhost'taki gibi görünmüyordu.
İnaktif, Disk Alanı, SCCM, TH, BSOD, Monitor dosyaları güncel gerçekçi
versiyonlarla değiştirildi; Lokasyon Mail Listesi ilk kez bundle'a eklendi.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/backend/demo-data/current/InaktifCihazlar_20260901000000.xlsx
+++ b/backend/demo-data/current/InaktifCihazlar_20260901000000.xlsx
@@ -441,16 +441,16 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>SYNPC001421</v>
+        <v>PFLRLBA3</v>
       </c>
       <c r="B2" t="str">
-        <v>Kullanıcı 23</v>
+        <v>Ali Yıldız</v>
       </c>
       <c r="C2" t="str">
-        <v>GENEL MUDURLUK (SENTETIK)</v>
+        <v>GENEL MUDURLUK</v>
       </c>
       <c r="D2" t="str">
-        <v>Sentetik ThinkPad SYN</v>
+        <v>Lenovo ThinkPad X1 Carbon</v>
       </c>
       <c r="E2" t="str">
         <v>TKAJ-AJET A.Ş.</v>
@@ -464,16 +464,16 @@
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>SYNMN000162</v>
+        <v>CN004XZ25</v>
       </c>
       <c r="B3" t="str">
-        <v>Kullanıcı 320</v>
+        <v>Okan Şahin</v>
       </c>
       <c r="C3" t="str">
         <v>SUBE-B</v>
       </c>
       <c r="D3" t="str">
-        <v>Sentetik Monitör Model</v>
+        <v>LG 24MK430H</v>
       </c>
       <c r="E3" t="str">
         <v>TKAO-THY A.O.</v>
@@ -487,16 +487,16 @@
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>SYNPC000346</v>
+        <v>PFAC9WYF</v>
       </c>
       <c r="B4" t="str">
-        <v>Kullanıcı 222</v>
+        <v>Büşra Demir</v>
       </c>
       <c r="C4" t="str">
         <v>SUBE-C</v>
       </c>
       <c r="D4" t="str">
-        <v>Sentetik ThinkPad SYN</v>
+        <v>HP EliteBook 840 G8</v>
       </c>
       <c r="E4" t="str">
         <v>TKAO-THY A.O.</v>
@@ -510,16 +510,16 @@
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>SYNPC000359</v>
+        <v>06CZTVL</v>
       </c>
       <c r="B5" t="str">
-        <v>Kullanıcı 1</v>
+        <v>Hüseyin Özdemir</v>
       </c>
       <c r="C5" t="str">
         <v>LOJISTIK MERKEZI</v>
       </c>
       <c r="D5" t="str">
-        <v>Sentetik OptiPlex SYN</v>
+        <v>Dell OptiPlex 5090</v>
       </c>
       <c r="E5" t="str">
         <v>TKAO-THY A.O.</v>
@@ -533,16 +533,16 @@
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>SYNMN000421</v>
+        <v>CN00CSVPQ</v>
       </c>
       <c r="B6" t="str">
-        <v>Kullanıcı 139</v>
+        <v>Zeynep Yıldız</v>
       </c>
       <c r="C6" t="str">
         <v>EGITIM MERKEZI</v>
       </c>
       <c r="D6" t="str">
-        <v>Sentetik Monitör Model</v>
+        <v>Dell U2419H</v>
       </c>
       <c r="E6" t="str">
         <v>TKAO-THY A.O.</v>
@@ -556,16 +556,16 @@
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>SYNPC001089</v>
+        <v>0AU6PJM</v>
       </c>
       <c r="B7" t="str">
-        <v>Kullanıcı 214</v>
+        <v>Barış Yıldırım</v>
       </c>
       <c r="C7" t="str">
         <v>SUBE-A</v>
       </c>
       <c r="D7" t="str">
-        <v>Sentetik OptiPlex SYN</v>
+        <v>Lenovo ThinkCentre M90</v>
       </c>
       <c r="E7" t="str">
         <v>TKAJ-AJET A.Ş.</v>
@@ -579,16 +579,16 @@
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>SYNMN000664</v>
+        <v>CN00L59R1</v>
       </c>
       <c r="B8" t="str">
-        <v>Kullanıcı 170</v>
+        <v>Cem Yılmaz</v>
       </c>
       <c r="C8" t="str">
         <v>MERKEZ BINA</v>
       </c>
       <c r="D8" t="str">
-        <v>Sentetik Monitör Model</v>
+        <v>Dell P2419H</v>
       </c>
       <c r="E8" t="str">
         <v>TKAJ-AJET A.Ş.</v>
@@ -602,16 +602,16 @@
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>SYNPC001126</v>
+        <v>PFYBZ1Z1</v>
       </c>
       <c r="B9" t="str">
-        <v>Kullanıcı 129</v>
+        <v>İpek Yıldız</v>
       </c>
       <c r="C9" t="str">
         <v>SAHA OFISI-1</v>
       </c>
       <c r="D9" t="str">
-        <v>Sentetik ThinkPad SYN</v>
+        <v>Lenovo ThinkPad X1 Carbon</v>
       </c>
       <c r="E9" t="str">
         <v>TKAO-THY A.O.</v>
@@ -625,16 +625,16 @@
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>SYNPC000491</v>
+        <v>PF5V6BS3</v>
       </c>
       <c r="B10" t="str">
-        <v>Kullanıcı 24</v>
+        <v>Elif Şahin</v>
       </c>
       <c r="C10" t="str">
         <v>SUBE-B</v>
       </c>
       <c r="D10" t="str">
-        <v>Sentetik ThinkPad SYN</v>
+        <v>Lenovo ThinkPad T14</v>
       </c>
       <c r="E10" t="str">
         <v>TKAJ-AJET A.Ş.</v>
@@ -648,16 +648,16 @@
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>SYNMN000046</v>
+        <v>CN001EERF</v>
       </c>
       <c r="B11" t="str">
-        <v>Kullanıcı 38</v>
+        <v>Sultan Demir</v>
       </c>
       <c r="C11" t="str">
         <v>EGITIM MERKEZI</v>
       </c>
       <c r="D11" t="str">
-        <v>Sentetik Monitör Model</v>
+        <v>LG 24MK430H</v>
       </c>
       <c r="E11" t="str">
         <v>TKAO-THY A.O.</v>
@@ -671,16 +671,16 @@
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>SYNPC001414</v>
+        <v>07FUY4Y</v>
       </c>
       <c r="B12" t="str">
-        <v>Kullanıcı 223</v>
+        <v>Şeyma Şahin</v>
       </c>
       <c r="C12" t="str">
         <v>SUBE-A</v>
       </c>
       <c r="D12" t="str">
-        <v>Sentetik ThinkPad SYN</v>
+        <v>Dell Latitude 5420</v>
       </c>
       <c r="E12" t="str">
         <v>TKAO-THY A.O.</v>
@@ -694,16 +694,16 @@
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>SYNMN000740</v>
+        <v>CN00NFLK5</v>
       </c>
       <c r="B13" t="str">
-        <v>Kullanıcı 151</v>
+        <v>Ali Özdemir</v>
       </c>
       <c r="C13" t="str">
         <v>MERKEZ BINA</v>
       </c>
       <c r="D13" t="str">
-        <v>Sentetik Monitör Model</v>
+        <v>Dell P2419H</v>
       </c>
       <c r="E13" t="str">
         <v>TKAO-THY A.O.</v>
@@ -717,16 +717,16 @@
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>SYNMN000187</v>
+        <v>CN005PQZS</v>
       </c>
       <c r="B14" t="str">
-        <v>Kullanıcı 106</v>
+        <v>Tolga Yılmaz</v>
       </c>
       <c r="C14" t="str">
         <v>LOJISTIK MERKEZI</v>
       </c>
       <c r="D14" t="str">
-        <v>Sentetik Monitör Model</v>
+        <v>Samsung S24R350</v>
       </c>
       <c r="E14" t="str">
         <v>TKAJ-AJET A.Ş.</v>
@@ -740,16 +740,16 @@
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>SYNMN000592</v>
+        <v>CN00HZ31Z</v>
       </c>
       <c r="B15" t="str">
-        <v>Kullanıcı 213</v>
+        <v>Hasan Aslan</v>
       </c>
       <c r="C15" t="str">
         <v>MERKEZ BINA</v>
       </c>
       <c r="D15" t="str">
-        <v>Sentetik Monitör Model</v>
+        <v>Dell P2419H</v>
       </c>
       <c r="E15" t="str">
         <v>TKAO-THY A.O.</v>
@@ -763,16 +763,16 @@
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>SYNMN000618</v>
+        <v>CN00JRW0V</v>
       </c>
       <c r="B16" t="str">
-        <v>Kullanıcı 235</v>
+        <v>Derya Kaya</v>
       </c>
       <c r="C16" t="str">
         <v>SUBE-C</v>
       </c>
       <c r="D16" t="str">
-        <v>Sentetik Monitör Model</v>
+        <v>LG 24MK430H</v>
       </c>
       <c r="E16" t="str">
         <v>TKAJ-AJET A.Ş.</v>
@@ -786,16 +786,16 @@
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>SYNMN000628</v>
+        <v>CN00K26DH</v>
       </c>
       <c r="B17" t="str">
-        <v>Kullanıcı 90</v>
+        <v>Selin Yıldırım</v>
       </c>
       <c r="C17" t="str">
         <v>SUBE-C</v>
       </c>
       <c r="D17" t="str">
-        <v>Sentetik Monitör Model</v>
+        <v>Dell P2419H</v>
       </c>
       <c r="E17" t="str">
         <v>TKAO-THY A.O.</v>
@@ -809,16 +809,16 @@
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>SYNPC001161</v>
+        <v>0EKBTGT</v>
       </c>
       <c r="B18" t="str">
-        <v>Kullanıcı 64</v>
+        <v>Şeyma Özdemir</v>
       </c>
       <c r="C18" t="str">
         <v>LOJISTIK MERKEZI</v>
       </c>
       <c r="D18" t="str">
-        <v>Sentetik OptiPlex SYN</v>
+        <v>Lenovo ThinkCentre M90</v>
       </c>
       <c r="E18" t="str">
         <v>TKAO-THY A.O.</v>
@@ -832,16 +832,16 @@
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>SYNPC000948</v>
+        <v>PFYN1A5L</v>
       </c>
       <c r="B19" t="str">
-        <v>Kullanıcı 92</v>
+        <v>Sultan Yılmaz</v>
       </c>
       <c r="C19" t="str">
         <v>SUBE-A</v>
       </c>
       <c r="D19" t="str">
-        <v>Sentetik ThinkPad SYN</v>
+        <v>Lenovo ThinkPad X1 Carbon</v>
       </c>
       <c r="E19" t="str">
         <v>TKAO-THY A.O.</v>
@@ -855,16 +855,16 @@
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>SYNMN000037</v>
+        <v>CN00155E2</v>
       </c>
       <c r="B20" t="str">
-        <v>Kullanıcı 113</v>
+        <v>Cansu Çelik</v>
       </c>
       <c r="C20" t="str">
         <v>SUBE-C</v>
       </c>
       <c r="D20" t="str">
-        <v>Sentetik Monitör Model</v>
+        <v>Dell U2419H</v>
       </c>
       <c r="E20" t="str">
         <v>TKAJ-AJET A.Ş.</v>
@@ -878,16 +878,16 @@
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>SYNPC001724</v>
+        <v>02NTG6Y</v>
       </c>
       <c r="B21" t="str">
-        <v>Kullanıcı 188</v>
+        <v>Gizem Yıldırım</v>
       </c>
       <c r="C21" t="str">
         <v>SUBE-B</v>
       </c>
       <c r="D21" t="str">
-        <v>Sentetik OptiPlex SYN</v>
+        <v>Dell OptiPlex 7090</v>
       </c>
       <c r="E21" t="str">
         <v>TKAJ-AJET A.Ş.</v>
@@ -901,16 +901,16 @@
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>SYNPC000394</v>
+        <v>PFEHA7Z9</v>
       </c>
       <c r="B22" t="str">
-        <v>Kullanıcı 46</v>
+        <v>Pınar Yıldız</v>
       </c>
       <c r="C22" t="str">
         <v>DEPO-1</v>
       </c>
       <c r="D22" t="str">
-        <v>Sentetik ThinkPad SYN</v>
+        <v>Dell Latitude 5420</v>
       </c>
       <c r="E22" t="str">
         <v>TKAO-THY A.O.</v>
@@ -924,16 +924,16 @@
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>SYNMN000446</v>
+        <v>CN00DJMMB</v>
       </c>
       <c r="B23" t="str">
-        <v>Kullanıcı 244</v>
+        <v>Pınar Öztürk</v>
       </c>
       <c r="C23" t="str">
         <v>SUBE-A</v>
       </c>
       <c r="D23" t="str">
-        <v>Sentetik Monitör Model</v>
+        <v>LG 24MK430H</v>
       </c>
       <c r="E23" t="str">
         <v>TKAJ-AJET A.Ş.</v>
@@ -947,16 +947,16 @@
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v>SYNPC000937</v>
+        <v>05AH8T5</v>
       </c>
       <c r="B24" t="str">
-        <v>Kullanıcı 211</v>
+        <v>Osman Yılmaz</v>
       </c>
       <c r="C24" t="str">
         <v>SAHA OFISI-2</v>
       </c>
       <c r="D24" t="str">
-        <v>Sentetik OptiPlex SYN</v>
+        <v>Lenovo ThinkCentre M90</v>
       </c>
       <c r="E24" t="str">
         <v>TKAO-THY A.O.</v>
@@ -970,16 +970,16 @@
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v>SYNPC001936</v>
+        <v>PFZR92HL</v>
       </c>
       <c r="B25" t="str">
-        <v>Kullanıcı 149</v>
+        <v>Meryem Şahin</v>
       </c>
       <c r="C25" t="str">
         <v>SAHA OFISI-1</v>
       </c>
       <c r="D25" t="str">
-        <v>Sentetik ThinkPad SYN</v>
+        <v>Lenovo ThinkPad X1 Carbon</v>
       </c>
       <c r="E25" t="str">
         <v>TKAJ-AJET A.Ş.</v>
@@ -993,16 +993,16 @@
     </row>
     <row r="26">
       <c r="A26" t="str">
-        <v>SYNPC001559</v>
+        <v>0FDX273</v>
       </c>
       <c r="B26" t="str">
-        <v>Kullanıcı 209</v>
+        <v>Ali Şahin</v>
       </c>
       <c r="C26" t="str">
         <v>LOJISTIK MERKEZI</v>
       </c>
       <c r="D26" t="str">
-        <v>Sentetik OptiPlex SYN</v>
+        <v>HP EliteDesk 800 G6</v>
       </c>
       <c r="E26" t="str">
         <v>TKAO-THY A.O.</v>
@@ -1016,16 +1016,16 @@
     </row>
     <row r="27">
       <c r="A27" t="str">
-        <v>SYNPC001147</v>
+        <v>0B01J0H</v>
       </c>
       <c r="B27" t="str">
-        <v>Kullanıcı 273</v>
+        <v>Tolga Kaya</v>
       </c>
       <c r="C27" t="str">
         <v>SAHA OFISI-1</v>
       </c>
       <c r="D27" t="str">
-        <v>Sentetik OptiPlex SYN</v>
+        <v>Lenovo ThinkCentre M90</v>
       </c>
       <c r="E27" t="str">
         <v>TKAJ-AJET A.Ş.</v>
@@ -1039,16 +1039,16 @@
     </row>
     <row r="28">
       <c r="A28" t="str">
-        <v>SYNMN000148</v>
+        <v>CN004HJJF</v>
       </c>
       <c r="B28" t="str">
-        <v>Kullanıcı 318</v>
+        <v>Hasan Aydın</v>
       </c>
       <c r="C28" t="str">
         <v>DEPO-1</v>
       </c>
       <c r="D28" t="str">
-        <v>Sentetik Monitör Model</v>
+        <v>Dell P2419H</v>
       </c>
       <c r="E28" t="str">
         <v>TKAO-THY A.O.</v>
@@ -1062,16 +1062,16 @@
     </row>
     <row r="29">
       <c r="A29" t="str">
-        <v>SYNPC001173</v>
+        <v>06SWW0U</v>
       </c>
       <c r="B29" t="str">
-        <v>Kullanıcı 194</v>
+        <v>Mehmet Yıldırım</v>
       </c>
       <c r="C29" t="str">
         <v>SUBE-A</v>
       </c>
       <c r="D29" t="str">
-        <v>Sentetik ThinkPad SYN</v>
+        <v>HP EliteBook 840 G8</v>
       </c>
       <c r="E29" t="str">
         <v>TKAJ-AJET A.Ş.</v>
@@ -1085,16 +1085,16 @@
     </row>
     <row r="30">
       <c r="A30" t="str">
-        <v>SYNMN000123</v>
+        <v>CN003RSLU</v>
       </c>
       <c r="B30" t="str">
-        <v>Kullanıcı 33</v>
+        <v>Yusuf Yıldırım</v>
       </c>
       <c r="C30" t="str">
         <v>EGITIM MERKEZI</v>
       </c>
       <c r="D30" t="str">
-        <v>Sentetik Monitör Model</v>
+        <v>Samsung S24R350</v>
       </c>
       <c r="E30" t="str">
         <v>TKAJ-AJET A.Ş.</v>
@@ -1108,16 +1108,16 @@
     </row>
     <row r="31">
       <c r="A31" t="str">
-        <v>SYNPC001849</v>
+        <v>0MN8FS1</v>
       </c>
       <c r="B31" t="str">
-        <v>Kullanıcı 153</v>
+        <v>Ahmet Yıldız</v>
       </c>
       <c r="C31" t="str">
         <v>LOJISTIK MERKEZI</v>
       </c>
       <c r="D31" t="str">
-        <v>Sentetik OptiPlex SYN</v>
+        <v>Lenovo ThinkCentre M90</v>
       </c>
       <c r="E31" t="str">
         <v>TKAO-THY A.O.</v>
@@ -1131,16 +1131,16 @@
     </row>
     <row r="32">
       <c r="A32" t="str">
-        <v>SYNPC000451</v>
+        <v>0D4N2YG</v>
       </c>
       <c r="B32" t="str">
-        <v>Kullanıcı 197</v>
+        <v>Hatice Demir</v>
       </c>
       <c r="C32" t="str">
         <v>SAHA OFISI-2</v>
       </c>
       <c r="D32" t="str">
-        <v>Sentetik OptiPlex SYN</v>
+        <v>Lenovo ThinkCentre M90</v>
       </c>
       <c r="E32" t="str">
         <v>TKAO-THY A.O.</v>
@@ -1154,16 +1154,16 @@
     </row>
     <row r="33">
       <c r="A33" t="str">
-        <v>SYNPC001673</v>
+        <v>PF1FXNC5</v>
       </c>
       <c r="B33" t="str">
-        <v>Kullanıcı 216</v>
+        <v>Serkan Aslan</v>
       </c>
       <c r="C33" t="str">
         <v>LOJISTIK MERKEZI</v>
       </c>
       <c r="D33" t="str">
-        <v>Sentetik ThinkPad SYN</v>
+        <v>Lenovo ThinkPad T14</v>
       </c>
       <c r="E33" t="str">
         <v>TKAO-THY A.O.</v>
@@ -1177,16 +1177,16 @@
     </row>
     <row r="34">
       <c r="A34" t="str">
-        <v>SYNPC001974</v>
+        <v>PFX61G8D</v>
       </c>
       <c r="B34" t="str">
-        <v>Kullanıcı 228</v>
+        <v>Mehmet Şahin</v>
       </c>
       <c r="C34" t="str">
         <v>MERKEZ BINA</v>
       </c>
       <c r="D34" t="str">
-        <v>Sentetik ThinkPad SYN</v>
+        <v>HP EliteBook 840 G8</v>
       </c>
       <c r="E34" t="str">
         <v>TKAJ-AJET A.Ş.</v>
@@ -1200,16 +1200,16 @@
     </row>
     <row r="35">
       <c r="A35" t="str">
-        <v>SYNMN000682</v>
+        <v>CN00LPUDT</v>
       </c>
       <c r="B35" t="str">
-        <v>Kullanıcı 126</v>
+        <v>Hasan Kaya</v>
       </c>
       <c r="C35" t="str">
         <v>LOJISTIK MERKEZI</v>
       </c>
       <c r="D35" t="str">
-        <v>Sentetik Monitör Model</v>
+        <v>LG 24MK430H</v>
       </c>
       <c r="E35" t="str">
         <v>TKAO-THY A.O.</v>
@@ -1223,16 +1223,16 @@
     </row>
     <row r="36">
       <c r="A36" t="str">
-        <v>SYNPC001267</v>
+        <v>014PY9X</v>
       </c>
       <c r="B36" t="str">
-        <v>Kullanıcı 257</v>
+        <v>Gizem Kaya</v>
       </c>
       <c r="C36" t="str">
         <v>DEPO-1</v>
       </c>
       <c r="D36" t="str">
-        <v>Sentetik OptiPlex SYN</v>
+        <v>HP EliteDesk 800 G6</v>
       </c>
       <c r="E36" t="str">
         <v>TKAO-THY A.O.</v>
@@ -1246,16 +1246,16 @@
     </row>
     <row r="37">
       <c r="A37" t="str">
-        <v>SYNPC001595</v>
+        <v>0LL4FWH</v>
       </c>
       <c r="B37" t="str">
-        <v>Kullanıcı 120</v>
+        <v>Derya Öztürk</v>
       </c>
       <c r="C37" t="str">
         <v>DEPO-1</v>
       </c>
       <c r="D37" t="str">
-        <v>Sentetik OptiPlex SYN</v>
+        <v>Lenovo ThinkCentre M90</v>
       </c>
       <c r="E37" t="str">
         <v>TKAO-THY A.O.</v>
@@ -1269,16 +1269,16 @@
     </row>
     <row r="38">
       <c r="A38" t="str">
-        <v>SYNPC000021</v>
+        <v>0HZ0WCX</v>
       </c>
       <c r="B38" t="str">
-        <v>Kullanıcı 309</v>
+        <v>Kemal Yılmaz</v>
       </c>
       <c r="C38" t="str">
         <v>SUBE-A</v>
       </c>
       <c r="D38" t="str">
-        <v>Sentetik OptiPlex SYN</v>
+        <v>HP EliteDesk 800 G6</v>
       </c>
       <c r="E38" t="str">
         <v>TKAO-THY A.O.</v>
@@ -1292,16 +1292,16 @@
     </row>
     <row r="39">
       <c r="A39" t="str">
-        <v>SYNMN000427</v>
+        <v>CN00CZ1XA</v>
       </c>
       <c r="B39" t="str">
-        <v>Kullanıcı 153</v>
+        <v>Ahmet Yıldız</v>
       </c>
       <c r="C39" t="str">
         <v>LOJISTIK MERKEZI</v>
       </c>
       <c r="D39" t="str">
-        <v>Sentetik Monitör Model</v>
+        <v>Samsung S24R350</v>
       </c>
       <c r="E39" t="str">
         <v>TKAO-THY A.O.</v>
@@ -1315,16 +1315,16 @@
     </row>
     <row r="40">
       <c r="A40" t="str">
-        <v>SYNPC000541</v>
+        <v>0AKRWNC</v>
       </c>
       <c r="B40" t="str">
-        <v>Kullanıcı 9</v>
+        <v>Emine Kaya</v>
       </c>
       <c r="C40" t="str">
-        <v>GENEL MUDURLUK (SENTETIK)</v>
+        <v>GENEL MUDURLUK</v>
       </c>
       <c r="D40" t="str">
-        <v>Sentetik OptiPlex SYN</v>
+        <v>HP EliteDesk 800 G6</v>
       </c>
       <c r="E40" t="str">
         <v>TKAJ-AJET A.Ş.</v>
@@ -1338,16 +1338,16 @@
     </row>
     <row r="41">
       <c r="A41" t="str">
-        <v>SYNPC000966</v>
+        <v>PF2MGCL6</v>
       </c>
       <c r="B41" t="str">
-        <v>Kullanıcı 149</v>
+        <v>Meryem Şahin</v>
       </c>
       <c r="C41" t="str">
         <v>SUBE-B</v>
       </c>
       <c r="D41" t="str">
-        <v>Sentetik ThinkPad SYN</v>
+        <v>Lenovo ThinkPad X1 Carbon</v>
       </c>
       <c r="E41" t="str">
         <v>TKAJ-AJET A.Ş.</v>
@@ -1361,16 +1361,16 @@
     </row>
     <row r="42">
       <c r="A42" t="str">
-        <v>SYNPC000041</v>
+        <v>PFNYNMMD</v>
       </c>
       <c r="B42" t="str">
-        <v>Kullanıcı 89</v>
+        <v>Şeyma Yılmaz</v>
       </c>
       <c r="C42" t="str">
         <v>SUBE-A</v>
       </c>
       <c r="D42" t="str">
-        <v>Sentetik ThinkPad SYN</v>
+        <v>HP EliteBook 840 G8</v>
       </c>
       <c r="E42" t="str">
         <v>TKAO-THY A.O.</v>
@@ -1384,16 +1384,16 @@
     </row>
     <row r="43">
       <c r="A43" t="str">
-        <v>SYNPC000328</v>
+        <v>PFJNSEGN</v>
       </c>
       <c r="B43" t="str">
-        <v>Kullanıcı 97</v>
+        <v>Şeyma Kaya</v>
       </c>
       <c r="C43" t="str">
         <v>SUBE-B</v>
       </c>
       <c r="D43" t="str">
-        <v>Sentetik ThinkPad SYN</v>
+        <v>Dell Latitude 5420</v>
       </c>
       <c r="E43" t="str">
         <v>TKAO-THY A.O.</v>
@@ -1407,16 +1407,16 @@
     </row>
     <row r="44">
       <c r="A44" t="str">
-        <v>SYNPC000802</v>
+        <v>0L2NP1C</v>
       </c>
       <c r="B44" t="str">
-        <v>Kullanıcı 316</v>
+        <v>Ayşe Aydın</v>
       </c>
       <c r="C44" t="str">
         <v>SUBE-A</v>
       </c>
       <c r="D44" t="str">
-        <v>Sentetik OptiPlex SYN</v>
+        <v>Lenovo ThinkCentre M90</v>
       </c>
       <c r="E44" t="str">
         <v>TKAO-THY A.O.</v>
@@ -1430,16 +1430,16 @@
     </row>
     <row r="45">
       <c r="A45" t="str">
-        <v>SYNPC001661</v>
+        <v>0GDL0ZF</v>
       </c>
       <c r="B45" t="str">
-        <v>Kullanıcı 203</v>
+        <v>Hüseyin Doğan</v>
       </c>
       <c r="C45" t="str">
         <v>SUBE-C</v>
       </c>
       <c r="D45" t="str">
-        <v>Sentetik OptiPlex SYN</v>
+        <v>HP EliteDesk 800 G6</v>
       </c>
       <c r="E45" t="str">
         <v>TKAO-THY A.O.</v>
@@ -1453,16 +1453,16 @@
     </row>
     <row r="46">
       <c r="A46" t="str">
-        <v>SYNPC000069</v>
+        <v>089J547</v>
       </c>
       <c r="B46" t="str">
-        <v>Kullanıcı 183</v>
+        <v>Yusuf Kaya</v>
       </c>
       <c r="C46" t="str">
         <v>SUBE-A</v>
       </c>
       <c r="D46" t="str">
-        <v>Sentetik OptiPlex SYN</v>
+        <v>Dell OptiPlex 7090</v>
       </c>
       <c r="E46" t="str">
         <v>TKAO-THY A.O.</v>
@@ -1476,16 +1476,16 @@
     </row>
     <row r="47">
       <c r="A47" t="str">
-        <v>SYNMN000652</v>
+        <v>CN00KSX9V</v>
       </c>
       <c r="B47" t="str">
-        <v>Kullanıcı 317</v>
+        <v>Onur Demir</v>
       </c>
       <c r="C47" t="str">
         <v>MERKEZ BINA</v>
       </c>
       <c r="D47" t="str">
-        <v>Sentetik Monitör Model</v>
+        <v>Dell P2419H</v>
       </c>
       <c r="E47" t="str">
         <v>TKAO-THY A.O.</v>
@@ -1499,16 +1499,16 @@
     </row>
     <row r="48">
       <c r="A48" t="str">
-        <v>SYNPC001364</v>
+        <v>0864BRH</v>
       </c>
       <c r="B48" t="str">
-        <v>Kullanıcı 59</v>
+        <v>Cansu Demir</v>
       </c>
       <c r="C48" t="str">
         <v>EGITIM MERKEZI</v>
       </c>
       <c r="D48" t="str">
-        <v>Sentetik OptiPlex SYN</v>
+        <v>Lenovo ThinkCentre M90</v>
       </c>
       <c r="E48" t="str">
         <v>TKAO-THY A.O.</v>
@@ -1522,16 +1522,16 @@
     </row>
     <row r="49">
       <c r="A49" t="str">
-        <v>SYNPC000946</v>
+        <v>0262TRM</v>
       </c>
       <c r="B49" t="str">
-        <v>Kullanıcı 203</v>
+        <v>Hüseyin Doğan</v>
       </c>
       <c r="C49" t="str">
         <v>LOJISTIK MERKEZI</v>
       </c>
       <c r="D49" t="str">
-        <v>Sentetik OptiPlex SYN</v>
+        <v>Dell OptiPlex 5090</v>
       </c>
       <c r="E49" t="str">
         <v>TKAO-THY A.O.</v>
@@ -1545,16 +1545,16 @@
     </row>
     <row r="50">
       <c r="A50" t="str">
-        <v>SYNPC000875</v>
+        <v>0HHSGR8</v>
       </c>
       <c r="B50" t="str">
-        <v>Kullanıcı 192</v>
+        <v>Zeynep Kaya</v>
       </c>
       <c r="C50" t="str">
         <v>LOJISTIK MERKEZI</v>
       </c>
       <c r="D50" t="str">
-        <v>Sentetik OptiPlex SYN</v>
+        <v>Lenovo ThinkCentre M90</v>
       </c>
       <c r="E50" t="str">
         <v>TKAO-THY A.O.</v>
@@ -1568,16 +1568,16 @@
     </row>
     <row r="51">
       <c r="A51" t="str">
-        <v>SYNPC000087</v>
+        <v>0BUUELH</v>
       </c>
       <c r="B51" t="str">
-        <v>Kullanıcı 7</v>
+        <v>Elif Yılmaz</v>
       </c>
       <c r="C51" t="str">
         <v>EGITIM MERKEZI</v>
       </c>
       <c r="D51" t="str">
-        <v>Sentetik OptiPlex SYN</v>
+        <v>HP EliteDesk 800 G6</v>
       </c>
       <c r="E51" t="str">
         <v>TKAJ-AJET A.Ş.</v>
@@ -1591,16 +1591,16 @@
     </row>
     <row r="52">
       <c r="A52" t="str">
-        <v>SYNMN000616</v>
+        <v>CN00JPTYB</v>
       </c>
       <c r="B52" t="str">
-        <v>Kullanıcı 209</v>
+        <v>Ali Şahin</v>
       </c>
       <c r="C52" t="str">
         <v>MERKEZ BINA</v>
       </c>
       <c r="D52" t="str">
-        <v>Sentetik Monitör Model</v>
+        <v>Dell P2419H</v>
       </c>
       <c r="E52" t="str">
         <v>TKAJ-AJET A.Ş.</v>
@@ -1614,16 +1614,16 @@
     </row>
     <row r="53">
       <c r="A53" t="str">
-        <v>SYNMN000320</v>
+        <v>CN009QSXZ</v>
       </c>
       <c r="B53" t="str">
-        <v>Kullanıcı 188</v>
+        <v>Gizem Yıldırım</v>
       </c>
       <c r="C53" t="str">
         <v>SUBE-B</v>
       </c>
       <c r="D53" t="str">
-        <v>Sentetik Monitör Model</v>
+        <v>Dell P2419H</v>
       </c>
       <c r="E53" t="str">
         <v>TKAJ-AJET A.Ş.</v>
@@ -1637,16 +1637,16 @@
     </row>
     <row r="54">
       <c r="A54" t="str">
-        <v>SYNMN000258</v>
+        <v>CN007UWMK</v>
       </c>
       <c r="B54" t="str">
-        <v>Kullanıcı 153</v>
+        <v>Ahmet Yıldız</v>
       </c>
       <c r="C54" t="str">
-        <v>GENEL MUDURLUK (SENTETIK)</v>
+        <v>GENEL MUDURLUK</v>
       </c>
       <c r="D54" t="str">
-        <v>Sentetik Monitör Model</v>
+        <v>LG 24MK430H</v>
       </c>
       <c r="E54" t="str">
         <v>TKAO-THY A.O.</v>
@@ -1660,16 +1660,16 @@
     </row>
     <row r="55">
       <c r="A55" t="str">
-        <v>SYNPC000385</v>
+        <v>0LVRNY0</v>
       </c>
       <c r="B55" t="str">
-        <v>Kullanıcı 183</v>
+        <v>Yusuf Kaya</v>
       </c>
       <c r="C55" t="str">
-        <v>GENEL MUDURLUK (SENTETIK)</v>
+        <v>GENEL MUDURLUK</v>
       </c>
       <c r="D55" t="str">
-        <v>Sentetik OptiPlex SYN</v>
+        <v>Dell OptiPlex 7090</v>
       </c>
       <c r="E55" t="str">
         <v>TKAJ-AJET A.Ş.</v>
@@ -1683,16 +1683,16 @@
     </row>
     <row r="56">
       <c r="A56" t="str">
-        <v>SYNPC001787</v>
+        <v>PFSZE0R5</v>
       </c>
       <c r="B56" t="str">
-        <v>Kullanıcı 120</v>
+        <v>Derya Öztürk</v>
       </c>
       <c r="C56" t="str">
         <v>MERKEZ BINA</v>
       </c>
       <c r="D56" t="str">
-        <v>Sentetik ThinkPad SYN</v>
+        <v>Lenovo ThinkPad X1 Carbon</v>
       </c>
       <c r="E56" t="str">
         <v>TKAJ-AJET A.Ş.</v>
@@ -1706,16 +1706,16 @@
     </row>
     <row r="57">
       <c r="A57" t="str">
-        <v>SYNMN000681</v>
+        <v>CN00LNTCJ</v>
       </c>
       <c r="B57" t="str">
-        <v>Kullanıcı 87</v>
+        <v>Onur Yıldız</v>
       </c>
       <c r="C57" t="str">
         <v>SAHA OFISI-2</v>
       </c>
       <c r="D57" t="str">
-        <v>Sentetik Monitör Model</v>
+        <v>Dell U2419H</v>
       </c>
       <c r="E57" t="str">
         <v>TKAO-THY A.O.</v>
@@ -1729,16 +1729,16 @@
     </row>
     <row r="58">
       <c r="A58" t="str">
-        <v>SYNPC000660</v>
+        <v>0LBPP08</v>
       </c>
       <c r="B58" t="str">
-        <v>Kullanıcı 210</v>
+        <v>Ali Çelik</v>
       </c>
       <c r="C58" t="str">
         <v>EGITIM MERKEZI</v>
       </c>
       <c r="D58" t="str">
-        <v>Sentetik OptiPlex SYN</v>
+        <v>Lenovo ThinkCentre M90</v>
       </c>
       <c r="E58" t="str">
         <v>TKAO-THY A.O.</v>
@@ -1752,16 +1752,16 @@
     </row>
     <row r="59">
       <c r="A59" t="str">
-        <v>SYNPC000166</v>
+        <v>PFHEK2E1</v>
       </c>
       <c r="B59" t="str">
-        <v>Kullanıcı 252</v>
+        <v>Aslı Demir</v>
       </c>
       <c r="C59" t="str">
-        <v>GENEL MUDURLUK (SENTETIK)</v>
+        <v>GENEL MUDURLUK</v>
       </c>
       <c r="D59" t="str">
-        <v>Sentetik ThinkPad SYN</v>
+        <v>Lenovo ThinkPad T14</v>
       </c>
       <c r="E59" t="str">
         <v>TKAO-THY A.O.</v>
@@ -1775,16 +1775,16 @@
     </row>
     <row r="60">
       <c r="A60" t="str">
-        <v>SYNPC000537</v>
+        <v>0H2WNAG</v>
       </c>
       <c r="B60" t="str">
-        <v>Kullanıcı 298</v>
+        <v>Aslı Yıldız</v>
       </c>
       <c r="C60" t="str">
         <v>DEPO-1</v>
       </c>
       <c r="D60" t="str">
-        <v>Sentetik OptiPlex SYN</v>
+        <v>HP EliteDesk 800 G6</v>
       </c>
       <c r="E60" t="str">
         <v>TKAO-THY A.O.</v>
@@ -1798,16 +1798,16 @@
     </row>
     <row r="61">
       <c r="A61" t="str">
-        <v>SYNPC000424</v>
+        <v>PFFQXFJG</v>
       </c>
       <c r="B61" t="str">
-        <v>Kullanıcı 237</v>
+        <v>Barış Yılmaz</v>
       </c>
       <c r="C61" t="str">
         <v>SAHA OFISI-1</v>
       </c>
       <c r="D61" t="str">
-        <v>Sentetik ThinkPad SYN</v>
+        <v>Lenovo ThinkPad X1 Carbon</v>
       </c>
       <c r="E61" t="str">
         <v>TKAO-THY A.O.</v>
@@ -1821,16 +1821,16 @@
     </row>
     <row r="62">
       <c r="A62" t="str">
-        <v>SYNPC001033</v>
+        <v>PF8Z4Y67</v>
       </c>
       <c r="B62" t="str">
-        <v>Kullanıcı 217</v>
+        <v>Mustafa Demir</v>
       </c>
       <c r="C62" t="str">
         <v>MERKEZ BINA</v>
       </c>
       <c r="D62" t="str">
-        <v>Sentetik ThinkPad SYN</v>
+        <v>HP EliteBook 840 G8</v>
       </c>
       <c r="E62" t="str">
         <v>TKAO-THY A.O.</v>
@@ -1844,16 +1844,16 @@
     </row>
     <row r="63">
       <c r="A63" t="str">
-        <v>SYNPC001945</v>
+        <v>PF88DULZ</v>
       </c>
       <c r="B63" t="str">
-        <v>Kullanıcı 218</v>
+        <v>Barış Yıldız</v>
       </c>
       <c r="C63" t="str">
         <v>DEPO-1</v>
       </c>
       <c r="D63" t="str">
-        <v>Sentetik ThinkPad SYN</v>
+        <v>HP EliteBook 840 G8</v>
       </c>
       <c r="E63" t="str">
         <v>TKAJ-AJET A.Ş.</v>
@@ -1867,16 +1867,16 @@
     </row>
     <row r="64">
       <c r="A64" t="str">
-        <v>SYNMN000752</v>
+        <v>CN00NTZ0B</v>
       </c>
       <c r="B64" t="str">
-        <v>Kullanıcı 55</v>
+        <v>Sultan Özdemir</v>
       </c>
       <c r="C64" t="str">
         <v>EGITIM MERKEZI</v>
       </c>
       <c r="D64" t="str">
-        <v>Sentetik Monitör Model</v>
+        <v>Dell P2419H</v>
       </c>
       <c r="E64" t="str">
         <v>TKAO-THY A.O.</v>
@@ -1890,16 +1890,16 @@
     </row>
     <row r="65">
       <c r="A65" t="str">
-        <v>SYNPC000880</v>
+        <v>PFF2E3MS</v>
       </c>
       <c r="B65" t="str">
-        <v>Kullanıcı 209</v>
+        <v>Ali Şahin</v>
       </c>
       <c r="C65" t="str">
         <v>EGITIM MERKEZI</v>
       </c>
       <c r="D65" t="str">
-        <v>Sentetik ThinkPad SYN</v>
+        <v>Lenovo ThinkPad T14</v>
       </c>
       <c r="E65" t="str">
         <v>TKAJ-AJET A.Ş.</v>
@@ -1913,16 +1913,16 @@
     </row>
     <row r="66">
       <c r="A66" t="str">
-        <v>SYNPC001304</v>
+        <v>PF7G2LVV</v>
       </c>
       <c r="B66" t="str">
-        <v>Kullanıcı 35</v>
+        <v>Büşra Aslan</v>
       </c>
       <c r="C66" t="str">
         <v>SUBE-C</v>
       </c>
       <c r="D66" t="str">
-        <v>Sentetik ThinkPad SYN</v>
+        <v>HP EliteBook 840 G8</v>
       </c>
       <c r="E66" t="str">
         <v>TKAO-THY A.O.</v>
@@ -1936,16 +1936,16 @@
     </row>
     <row r="67">
       <c r="A67" t="str">
-        <v>SYNMN000072</v>
+        <v>CN00277QB</v>
       </c>
       <c r="B67" t="str">
-        <v>Kullanıcı 256</v>
+        <v>Serkan Kaya</v>
       </c>
       <c r="C67" t="str">
         <v>SUBE-C</v>
       </c>
       <c r="D67" t="str">
-        <v>Sentetik Monitör Model</v>
+        <v>Dell P2419H</v>
       </c>
       <c r="E67" t="str">
         <v>TKAO-THY A.O.</v>
@@ -1959,16 +1959,16 @@
     </row>
     <row r="68">
       <c r="A68" t="str">
-        <v>SYNMN000124</v>
+        <v>CN003STN3</v>
       </c>
       <c r="B68" t="str">
-        <v>Kullanıcı 78</v>
+        <v>Ali Yılmaz</v>
       </c>
       <c r="C68" t="str">
         <v>SAHA OFISI-1</v>
       </c>
       <c r="D68" t="str">
-        <v>Sentetik Monitör Model</v>
+        <v>Dell P2419H</v>
       </c>
       <c r="E68" t="str">
         <v>TKAJ-AJET A.Ş.</v>
@@ -1982,16 +1982,16 @@
     </row>
     <row r="69">
       <c r="A69" t="str">
-        <v>SYNMN000718</v>
+        <v>CN00MSXRB</v>
       </c>
       <c r="B69" t="str">
-        <v>Kullanıcı 70</v>
+        <v>Osman Aydın</v>
       </c>
       <c r="C69" t="str">
         <v>SUBE-C</v>
       </c>
       <c r="D69" t="str">
-        <v>Sentetik Monitör Model</v>
+        <v>LG 24MK430H</v>
       </c>
       <c r="E69" t="str">
         <v>TKAJ-AJET A.Ş.</v>
@@ -2005,16 +2005,16 @@
     </row>
     <row r="70">
       <c r="A70" t="str">
-        <v>SYNPC001148</v>
+        <v>03DFF0E</v>
       </c>
       <c r="B70" t="str">
-        <v>Kullanıcı 282</v>
+        <v>Onur Yıldırım</v>
       </c>
       <c r="C70" t="str">
-        <v>GENEL MUDURLUK (SENTETIK)</v>
+        <v>GENEL MUDURLUK</v>
       </c>
       <c r="D70" t="str">
-        <v>Sentetik OptiPlex SYN</v>
+        <v>Dell OptiPlex 7090</v>
       </c>
       <c r="E70" t="str">
         <v>TKAO-THY A.O.</v>
@@ -2028,16 +2028,16 @@
     </row>
     <row r="71">
       <c r="A71" t="str">
-        <v>SYNPC001352</v>
+        <v>0J73429</v>
       </c>
       <c r="B71" t="str">
-        <v>Kullanıcı 217</v>
+        <v>Mustafa Demir</v>
       </c>
       <c r="C71" t="str">
-        <v>GENEL MUDURLUK (SENTETIK)</v>
+        <v>GENEL MUDURLUK</v>
       </c>
       <c r="D71" t="str">
-        <v>Sentetik OptiPlex SYN</v>
+        <v>Dell OptiPlex 5090</v>
       </c>
       <c r="E71" t="str">
         <v>TKAJ-AJET A.Ş.</v>
@@ -2051,16 +2051,16 @@
     </row>
     <row r="72">
       <c r="A72" t="str">
-        <v>SYNMN000315</v>
+        <v>CN009KMRN</v>
       </c>
       <c r="B72" t="str">
-        <v>Kullanıcı 147</v>
+        <v>Onur Kaya</v>
       </c>
       <c r="C72" t="str">
         <v>SAHA OFISI-2</v>
       </c>
       <c r="D72" t="str">
-        <v>Sentetik Monitör Model</v>
+        <v>Samsung S24R350</v>
       </c>
       <c r="E72" t="str">
         <v>TKAO-THY A.O.</v>
@@ -2074,16 +2074,16 @@
     </row>
     <row r="73">
       <c r="A73" t="str">
-        <v>SYNPC000520</v>
+        <v>03GMLHE</v>
       </c>
       <c r="B73" t="str">
-        <v>Kullanıcı 289</v>
+        <v>Gizem Yıldız</v>
       </c>
       <c r="C73" t="str">
         <v>DEPO-1</v>
       </c>
       <c r="D73" t="str">
-        <v>Sentetik ThinkPad SYN</v>
+        <v>Lenovo ThinkPad X1 Carbon</v>
       </c>
       <c r="E73" t="str">
         <v>TKAJ-AJET A.Ş.</v>
@@ -2097,16 +2097,16 @@
     </row>
     <row r="74">
       <c r="A74" t="str">
-        <v>SYNPC001878</v>
+        <v>0F6KYXK</v>
       </c>
       <c r="B74" t="str">
-        <v>Kullanıcı 71</v>
+        <v>Osman Şahin</v>
       </c>
       <c r="C74" t="str">
         <v>SUBE-B</v>
       </c>
       <c r="D74" t="str">
-        <v>Sentetik OptiPlex SYN</v>
+        <v>HP EliteDesk 800 G6</v>
       </c>
       <c r="E74" t="str">
         <v>TKAJ-AJET A.Ş.</v>
@@ -2120,16 +2120,16 @@
     </row>
     <row r="75">
       <c r="A75" t="str">
-        <v>SYNPC000745</v>
+        <v>09CRULG</v>
       </c>
       <c r="B75" t="str">
-        <v>Kullanıcı 175</v>
+        <v>İpek Şahin</v>
       </c>
       <c r="C75" t="str">
         <v>EGITIM MERKEZI</v>
       </c>
       <c r="D75" t="str">
-        <v>Sentetik OptiPlex SYN</v>
+        <v>HP EliteDesk 800 G6</v>
       </c>
       <c r="E75" t="str">
         <v>TKAJ-AJET A.Ş.</v>
@@ -2143,16 +2143,16 @@
     </row>
     <row r="76">
       <c r="A76" t="str">
-        <v>SYNMN000694</v>
+        <v>CN00M26UZ</v>
       </c>
       <c r="B76" t="str">
-        <v>Kullanıcı 309</v>
+        <v>Kemal Yılmaz</v>
       </c>
       <c r="C76" t="str">
         <v>SAHA OFISI-1</v>
       </c>
       <c r="D76" t="str">
-        <v>Sentetik Monitör Model</v>
+        <v>LG 24MK430H</v>
       </c>
       <c r="E76" t="str">
         <v>TKAO-THY A.O.</v>
@@ -2166,16 +2166,16 @@
     </row>
     <row r="77">
       <c r="A77" t="str">
-        <v>SYNMN000544</v>
+        <v>CN00GHM99</v>
       </c>
       <c r="B77" t="str">
-        <v>Kullanıcı 109</v>
+        <v>Nazlı Yıldırım</v>
       </c>
       <c r="C77" t="str">
         <v>EGITIM MERKEZI</v>
       </c>
       <c r="D77" t="str">
-        <v>Sentetik Monitör Model</v>
+        <v>Dell P2419H</v>
       </c>
       <c r="E77" t="str">
         <v>TKAO-THY A.O.</v>
@@ -2189,16 +2189,16 @@
     </row>
     <row r="78">
       <c r="A78" t="str">
-        <v>SYNPC001132</v>
+        <v>0E7VSER</v>
       </c>
       <c r="B78" t="str">
-        <v>Kullanıcı 53</v>
+        <v>Emine Şahin</v>
       </c>
       <c r="C78" t="str">
         <v>SAHA OFISI-2</v>
       </c>
       <c r="D78" t="str">
-        <v>Sentetik OptiPlex SYN</v>
+        <v>Lenovo ThinkCentre M90</v>
       </c>
       <c r="E78" t="str">
         <v>TKAO-THY A.O.</v>
@@ -2212,16 +2212,16 @@
     </row>
     <row r="79">
       <c r="A79" t="str">
-        <v>SYNMN000551</v>
+        <v>CN00GQUJ4</v>
       </c>
       <c r="B79" t="str">
-        <v>Kullanıcı 61</v>
+        <v>Selin Kaya</v>
       </c>
       <c r="C79" t="str">
         <v>MERKEZ BINA</v>
       </c>
       <c r="D79" t="str">
-        <v>Sentetik Monitör Model</v>
+        <v>Samsung S24R350</v>
       </c>
       <c r="E79" t="str">
         <v>TKAO-THY A.O.</v>
@@ -2235,16 +2235,16 @@
     </row>
     <row r="80">
       <c r="A80" t="str">
-        <v>SYNMN000307</v>
+        <v>CN009BDFJ</v>
       </c>
       <c r="B80" t="str">
-        <v>Kullanıcı 186</v>
+        <v>Derya Demir</v>
       </c>
       <c r="C80" t="str">
         <v>SAHA OFISI-1</v>
       </c>
       <c r="D80" t="str">
-        <v>Sentetik Monitör Model</v>
+        <v>Samsung S24R350</v>
       </c>
       <c r="E80" t="str">
         <v>TKAJ-AJET A.Ş.</v>
@@ -2258,16 +2258,16 @@
     </row>
     <row r="81">
       <c r="A81" t="str">
-        <v>SYNMN000126</v>
+        <v>CN003UVQM</v>
       </c>
       <c r="B81" t="str">
-        <v>Kullanıcı 156</v>
+        <v>Ozan Kaya</v>
       </c>
       <c r="C81" t="str">
         <v>SAHA OFISI-2</v>
       </c>
       <c r="D81" t="str">
-        <v>Sentetik Monitör Model</v>
+        <v>LG 24MK430H</v>
       </c>
       <c r="E81" t="str">
         <v>TKAO-THY A.O.</v>
@@ -2281,16 +2281,16 @@
     </row>
     <row r="82">
       <c r="A82" t="str">
-        <v>SYNPC000788</v>
+        <v>04Z17R3</v>
       </c>
       <c r="B82" t="str">
-        <v>Kullanıcı 59</v>
+        <v>Cansu Demir</v>
       </c>
       <c r="C82" t="str">
         <v>MERKEZ BINA</v>
       </c>
       <c r="D82" t="str">
-        <v>Sentetik OptiPlex SYN</v>
+        <v>Dell OptiPlex 7090</v>
       </c>
       <c r="E82" t="str">
         <v>TKAO-THY A.O.</v>
@@ -2304,16 +2304,16 @@
     </row>
     <row r="83">
       <c r="A83" t="str">
-        <v>SYNMN000750</v>
+        <v>CN00NRWXT</v>
       </c>
       <c r="B83" t="str">
-        <v>Kullanıcı 45</v>
+        <v>Emre Doğan</v>
       </c>
       <c r="C83" t="str">
         <v>EGITIM MERKEZI</v>
       </c>
       <c r="D83" t="str">
-        <v>Sentetik Monitör Model</v>
+        <v>LG 24MK430H</v>
       </c>
       <c r="E83" t="str">
         <v>TKAO-THY A.O.</v>
@@ -2327,16 +2327,16 @@
     </row>
     <row r="84">
       <c r="A84" t="str">
-        <v>SYNPC001750</v>
+        <v>05QEAYD</v>
       </c>
       <c r="B84" t="str">
-        <v>Kullanıcı 303</v>
+        <v>Serkan Yıldırım</v>
       </c>
       <c r="C84" t="str">
-        <v>GENEL MUDURLUK (SENTETIK)</v>
+        <v>GENEL MUDURLUK</v>
       </c>
       <c r="D84" t="str">
-        <v>Sentetik ThinkPad SYN</v>
+        <v>Lenovo ThinkPad X1 Carbon</v>
       </c>
       <c r="E84" t="str">
         <v>TKAO-THY A.O.</v>
@@ -2350,16 +2350,16 @@
     </row>
     <row r="85">
       <c r="A85" t="str">
-        <v>SYNPC001149</v>
+        <v>0HT61X1</v>
       </c>
       <c r="B85" t="str">
-        <v>Kullanıcı 79</v>
+        <v>Ozan Çelik</v>
       </c>
       <c r="C85" t="str">
         <v>SUBE-C</v>
       </c>
       <c r="D85" t="str">
-        <v>Sentetik OptiPlex SYN</v>
+        <v>Dell OptiPlex 5090</v>
       </c>
       <c r="E85" t="str">
         <v>TKAJ-AJET A.Ş.</v>
@@ -2373,16 +2373,16 @@
     </row>
     <row r="86">
       <c r="A86" t="str">
-        <v>SYNPC000836</v>
+        <v>PFN5BDKS</v>
       </c>
       <c r="B86" t="str">
-        <v>Kullanıcı 114</v>
+        <v>Emine Yıldırım</v>
       </c>
       <c r="C86" t="str">
         <v>DEPO-1</v>
       </c>
       <c r="D86" t="str">
-        <v>Sentetik ThinkPad SYN</v>
+        <v>Lenovo ThinkPad T14</v>
       </c>
       <c r="E86" t="str">
         <v>TKAO-THY A.O.</v>
@@ -2396,16 +2396,16 @@
     </row>
     <row r="87">
       <c r="A87" t="str">
-        <v>SYNPC001399</v>
+        <v>PF4J7MXP</v>
       </c>
       <c r="B87" t="str">
-        <v>Kullanıcı 143</v>
+        <v>Tolga Özdemir</v>
       </c>
       <c r="C87" t="str">
-        <v>GENEL MUDURLUK (SENTETIK)</v>
+        <v>GENEL MUDURLUK</v>
       </c>
       <c r="D87" t="str">
-        <v>Sentetik ThinkPad SYN</v>
+        <v>Dell Latitude 5420</v>
       </c>
       <c r="E87" t="str">
         <v>TKAJ-AJET A.Ş.</v>
@@ -2419,16 +2419,16 @@
     </row>
     <row r="88">
       <c r="A88" t="str">
-        <v>SYNPC001498</v>
+        <v>PF7BML8H</v>
       </c>
       <c r="B88" t="str">
-        <v>Kullanıcı 225</v>
+        <v>Şeyma Yıldırım</v>
       </c>
       <c r="C88" t="str">
         <v>EGITIM MERKEZI</v>
       </c>
       <c r="D88" t="str">
-        <v>Sentetik ThinkPad SYN</v>
+        <v>Dell Latitude 5420</v>
       </c>
       <c r="E88" t="str">
         <v>TKAO-THY A.O.</v>
@@ -2442,16 +2442,16 @@
     </row>
     <row r="89">
       <c r="A89" t="str">
-        <v>SYNPC001314</v>
+        <v>PFD6BH4V</v>
       </c>
       <c r="B89" t="str">
-        <v>Kullanıcı 220</v>
+        <v>Ozan Kılıç</v>
       </c>
       <c r="C89" t="str">
         <v>SAHA OFISI-2</v>
       </c>
       <c r="D89" t="str">
-        <v>Sentetik ThinkPad SYN</v>
+        <v>Lenovo ThinkPad T14</v>
       </c>
       <c r="E89" t="str">
         <v>TKAO-THY A.O.</v>
@@ -2465,16 +2465,16 @@
     </row>
     <row r="90">
       <c r="A90" t="str">
-        <v>SYNPC000425</v>
+        <v>PF3GZULP</v>
       </c>
       <c r="B90" t="str">
-        <v>Kullanıcı 230</v>
+        <v>Merve Şahin</v>
       </c>
       <c r="C90" t="str">
         <v>SUBE-C</v>
       </c>
       <c r="D90" t="str">
-        <v>Sentetik ThinkPad SYN</v>
+        <v>Dell Latitude 5420</v>
       </c>
       <c r="E90" t="str">
         <v>TKAJ-AJET A.Ş.</v>
@@ -2488,16 +2488,16 @@
     </row>
     <row r="91">
       <c r="A91" t="str">
-        <v>SYNPC001804</v>
+        <v>00XCV0D</v>
       </c>
       <c r="B91" t="str">
-        <v>Kullanıcı 273</v>
+        <v>Tolga Kaya</v>
       </c>
       <c r="C91" t="str">
         <v>SUBE-A</v>
       </c>
       <c r="D91" t="str">
-        <v>Sentetik OptiPlex SYN</v>
+        <v>Dell OptiPlex 5090</v>
       </c>
       <c r="E91" t="str">
         <v>TKAO-THY A.O.</v>
@@ -2511,16 +2511,16 @@
     </row>
     <row r="92">
       <c r="A92" t="str">
-        <v>SYNPC001481</v>
+        <v>PFUV3RQH</v>
       </c>
       <c r="B92" t="str">
-        <v>Kullanıcı 179</v>
+        <v>Hüseyin Demir</v>
       </c>
       <c r="C92" t="str">
         <v>SUBE-A</v>
       </c>
       <c r="D92" t="str">
-        <v>Sentetik ThinkPad SYN</v>
+        <v>Lenovo ThinkPad T14</v>
       </c>
       <c r="E92" t="str">
         <v>TKAO-THY A.O.</v>
@@ -2534,16 +2534,16 @@
     </row>
     <row r="93">
       <c r="A93" t="str">
-        <v>SYNPC000329</v>
+        <v>PF6DUTJV</v>
       </c>
       <c r="B93" t="str">
-        <v>Kullanıcı 262</v>
+        <v>Emre Şahin</v>
       </c>
       <c r="C93" t="str">
         <v>SAHA OFISI-2</v>
       </c>
       <c r="D93" t="str">
-        <v>Sentetik ThinkPad SYN</v>
+        <v>HP EliteBook 840 G8</v>
       </c>
       <c r="E93" t="str">
         <v>TKAJ-AJET A.Ş.</v>
@@ -2557,16 +2557,16 @@
     </row>
     <row r="94">
       <c r="A94" t="str">
-        <v>SYNMN000432</v>
+        <v>CN00D473M</v>
       </c>
       <c r="B94" t="str">
-        <v>Kullanıcı 179</v>
+        <v>Hüseyin Demir</v>
       </c>
       <c r="C94" t="str">
         <v>SUBE-A</v>
       </c>
       <c r="D94" t="str">
-        <v>Sentetik Monitör Model</v>
+        <v>Dell P2419H</v>
       </c>
       <c r="E94" t="str">
         <v>TKAO-THY A.O.</v>
@@ -2580,16 +2580,16 @@
     </row>
     <row r="95">
       <c r="A95" t="str">
-        <v>SYNPC000719</v>
+        <v>0GLX48Z</v>
       </c>
       <c r="B95" t="str">
-        <v>Kullanıcı 53</v>
+        <v>Emine Şahin</v>
       </c>
       <c r="C95" t="str">
         <v>SUBE-A</v>
       </c>
       <c r="D95" t="str">
-        <v>Sentetik OptiPlex SYN</v>
+        <v>Lenovo ThinkCentre M90</v>
       </c>
       <c r="E95" t="str">
         <v>TKAO-THY A.O.</v>
@@ -2603,16 +2603,16 @@
     </row>
     <row r="96">
       <c r="A96" t="str">
-        <v>SYNPC000278</v>
+        <v>PFPZUVL8</v>
       </c>
       <c r="B96" t="str">
-        <v>Kullanıcı 280</v>
+        <v>Emine Çelik</v>
       </c>
       <c r="C96" t="str">
-        <v>GENEL MUDURLUK (SENTETIK)</v>
+        <v>GENEL MUDURLUK</v>
       </c>
       <c r="D96" t="str">
-        <v>Sentetik ThinkPad SYN</v>
+        <v>Lenovo ThinkPad X1 Carbon</v>
       </c>
       <c r="E96" t="str">
         <v>TKAJ-AJET A.Ş.</v>
@@ -2626,16 +2626,16 @@
     </row>
     <row r="97">
       <c r="A97" t="str">
-        <v>SYNPC000600</v>
+        <v>PFJ5Q26A</v>
       </c>
       <c r="B97" t="str">
-        <v>Kullanıcı 167</v>
+        <v>Onur Çelik</v>
       </c>
       <c r="C97" t="str">
         <v>SUBE-B</v>
       </c>
       <c r="D97" t="str">
-        <v>Sentetik ThinkPad SYN</v>
+        <v>Dell Latitude 5420</v>
       </c>
       <c r="E97" t="str">
         <v>TKAO-THY A.O.</v>
@@ -2649,16 +2649,16 @@
     </row>
     <row r="98">
       <c r="A98" t="str">
-        <v>SYNPC000761</v>
+        <v>0DD2VUR</v>
       </c>
       <c r="B98" t="str">
-        <v>Kullanıcı 120</v>
+        <v>Derya Öztürk</v>
       </c>
       <c r="C98" t="str">
         <v>DEPO-1</v>
       </c>
       <c r="D98" t="str">
-        <v>Sentetik ThinkPad SYN</v>
+        <v>Lenovo ThinkPad X1 Carbon</v>
       </c>
       <c r="E98" t="str">
         <v>TKAJ-AJET A.Ş.</v>
@@ -2672,16 +2672,16 @@
     </row>
     <row r="99">
       <c r="A99" t="str">
-        <v>SYNPC000919</v>
+        <v>0DQJWWT</v>
       </c>
       <c r="B99" t="str">
-        <v>Kullanıcı 220</v>
+        <v>Ozan Kılıç</v>
       </c>
       <c r="C99" t="str">
         <v>SUBE-C</v>
       </c>
       <c r="D99" t="str">
-        <v>Sentetik ThinkPad SYN</v>
+        <v>HP EliteBook 840 G8</v>
       </c>
       <c r="E99" t="str">
         <v>TKAJ-AJET A.Ş.</v>
@@ -2695,16 +2695,16 @@
     </row>
     <row r="100">
       <c r="A100" t="str">
-        <v>SYNMN000775</v>
+        <v>CN00PHNVE</v>
       </c>
       <c r="B100" t="str">
-        <v>Kullanıcı 197</v>
+        <v>Hatice Demir</v>
       </c>
       <c r="C100" t="str">
-        <v>GENEL MUDURLUK (SENTETIK)</v>
+        <v>GENEL MUDURLUK</v>
       </c>
       <c r="D100" t="str">
-        <v>Sentetik Monitör Model</v>
+        <v>Samsung S24R350</v>
       </c>
       <c r="E100" t="str">
         <v>TKAJ-AJET A.Ş.</v>
@@ -2718,16 +2718,16 @@
     </row>
     <row r="101">
       <c r="A101" t="str">
-        <v>SYNPC001055</v>
+        <v>08CQAM7</v>
       </c>
       <c r="B101" t="str">
-        <v>Kullanıcı 71</v>
+        <v>Osman Şahin</v>
       </c>
       <c r="C101" t="str">
         <v>MERKEZ BINA</v>
       </c>
       <c r="D101" t="str">
-        <v>Sentetik OptiPlex SYN</v>
+        <v>HP EliteDesk 800 G6</v>
       </c>
       <c r="E101" t="str">
         <v>TKAJ-AJET A.Ş.</v>
@@ -2741,16 +2741,16 @@
     </row>
     <row r="102">
       <c r="A102" t="str">
-        <v>SYNPC000562</v>
+        <v>0ENHYZT</v>
       </c>
       <c r="B102" t="str">
-        <v>Kullanıcı 19</v>
+        <v>Şeyma Aydın</v>
       </c>
       <c r="C102" t="str">
         <v>MERKEZ BINA</v>
       </c>
       <c r="D102" t="str">
-        <v>Sentetik ThinkPad SYN</v>
+        <v>Lenovo ThinkPad T14</v>
       </c>
       <c r="E102" t="str">
         <v>TKAO-THY A.O.</v>
@@ -2764,16 +2764,16 @@
     </row>
     <row r="103">
       <c r="A103" t="str">
-        <v>SYNPC000434</v>
+        <v>PF0Q40S9</v>
       </c>
       <c r="B103" t="str">
-        <v>Kullanıcı 215</v>
+        <v>Murat Yıldırım</v>
       </c>
       <c r="C103" t="str">
         <v>SUBE-B</v>
       </c>
       <c r="D103" t="str">
-        <v>Sentetik ThinkPad SYN</v>
+        <v>Lenovo ThinkPad X1 Carbon</v>
       </c>
       <c r="E103" t="str">
         <v>TKAO-THY A.O.</v>
@@ -2787,16 +2787,16 @@
     </row>
     <row r="104">
       <c r="A104" t="str">
-        <v>SYNPC000665</v>
+        <v>PFW7MK1B</v>
       </c>
       <c r="B104" t="str">
-        <v>Kullanıcı 125</v>
+        <v>Mustafa Kaya</v>
       </c>
       <c r="C104" t="str">
         <v>SAHA OFISI-2</v>
       </c>
       <c r="D104" t="str">
-        <v>Sentetik ThinkPad SYN</v>
+        <v>Lenovo ThinkPad X1 Carbon</v>
       </c>
       <c r="E104" t="str">
         <v>TKAJ-AJET A.Ş.</v>
@@ -2810,16 +2810,16 @@
     </row>
     <row r="105">
       <c r="A105" t="str">
-        <v>SYNPC000097</v>
+        <v>02MB7DA</v>
       </c>
       <c r="B105" t="str">
-        <v>Kullanıcı 97</v>
+        <v>Şeyma Kaya</v>
       </c>
       <c r="C105" t="str">
         <v>DEPO-1</v>
       </c>
       <c r="D105" t="str">
-        <v>Sentetik OptiPlex SYN</v>
+        <v>HP EliteDesk 800 G6</v>
       </c>
       <c r="E105" t="str">
         <v>TKAO-THY A.O.</v>
@@ -2833,16 +2833,16 @@
     </row>
     <row r="106">
       <c r="A106" t="str">
-        <v>SYNPC000528</v>
+        <v>PFFJWBFP</v>
       </c>
       <c r="B106" t="str">
-        <v>Kullanıcı 77</v>
+        <v>Mustafa Yılmaz</v>
       </c>
       <c r="C106" t="str">
         <v>SAHA OFISI-1</v>
       </c>
       <c r="D106" t="str">
-        <v>Sentetik ThinkPad SYN</v>
+        <v>Lenovo ThinkPad X1 Carbon</v>
       </c>
       <c r="E106" t="str">
         <v>TKAJ-AJET A.Ş.</v>
@@ -2856,16 +2856,16 @@
     </row>
     <row r="107">
       <c r="A107" t="str">
-        <v>SYNPC000000</v>
+        <v>0EDQLWM</v>
       </c>
       <c r="B107" t="str">
-        <v>Kullanıcı 117</v>
+        <v>Ahmet Yılmaz</v>
       </c>
       <c r="C107" t="str">
         <v>SUBE-C</v>
       </c>
       <c r="D107" t="str">
-        <v>Sentetik OptiPlex SYN</v>
+        <v>Dell OptiPlex 7090</v>
       </c>
       <c r="E107" t="str">
         <v>TKAO-THY A.O.</v>
@@ -2879,16 +2879,16 @@
     </row>
     <row r="108">
       <c r="A108" t="str">
-        <v>SYNPC001374</v>
+        <v>0GPC5C5</v>
       </c>
       <c r="B108" t="str">
-        <v>Kullanıcı 301</v>
+        <v>Merve Yıldız</v>
       </c>
       <c r="C108" t="str">
-        <v>GENEL MUDURLUK (SENTETIK)</v>
+        <v>GENEL MUDURLUK</v>
       </c>
       <c r="D108" t="str">
-        <v>Sentetik OptiPlex SYN</v>
+        <v>Lenovo ThinkCentre M90</v>
       </c>
       <c r="E108" t="str">
         <v>TKAO-THY A.O.</v>
@@ -2902,16 +2902,16 @@
     </row>
     <row r="109">
       <c r="A109" t="str">
-        <v>SYNPC001546</v>
+        <v>0G7CMAN</v>
       </c>
       <c r="B109" t="str">
-        <v>Kullanıcı 146</v>
+        <v>Fatma Arslan</v>
       </c>
       <c r="C109" t="str">
         <v>SAHA OFISI-1</v>
       </c>
       <c r="D109" t="str">
-        <v>Sentetik OptiPlex SYN</v>
+        <v>Dell OptiPlex 7090</v>
       </c>
       <c r="E109" t="str">
         <v>TKAJ-AJET A.Ş.</v>
@@ -2925,16 +2925,16 @@
     </row>
     <row r="110">
       <c r="A110" t="str">
-        <v>SYNMN000524</v>
+        <v>CN00FX0HZ</v>
       </c>
       <c r="B110" t="str">
-        <v>Kullanıcı 260</v>
+        <v>Onur Özdemir</v>
       </c>
       <c r="C110" t="str">
         <v>SUBE-A</v>
       </c>
       <c r="D110" t="str">
-        <v>Sentetik Monitör Model</v>
+        <v>Dell P2419H</v>
       </c>
       <c r="E110" t="str">
         <v>TKAJ-AJET A.Ş.</v>
@@ -2948,16 +2948,16 @@
     </row>
     <row r="111">
       <c r="A111" t="str">
-        <v>SYNPC001703</v>
+        <v>07HJUUA</v>
       </c>
       <c r="B111" t="str">
-        <v>Kullanıcı 132</v>
+        <v>Okan Demir</v>
       </c>
       <c r="C111" t="str">
         <v>SUBE-C</v>
       </c>
       <c r="D111" t="str">
-        <v>Sentetik OptiPlex SYN</v>
+        <v>Dell OptiPlex 5090</v>
       </c>
       <c r="E111" t="str">
         <v>TKAJ-AJET A.Ş.</v>
@@ -2971,16 +2971,16 @@
     </row>
     <row r="112">
       <c r="A112" t="str">
-        <v>SYNMN000504</v>
+        <v>CN00FADSP</v>
       </c>
       <c r="B112" t="str">
-        <v>Kullanıcı 149</v>
+        <v>Meryem Şahin</v>
       </c>
       <c r="C112" t="str">
         <v>SUBE-B</v>
       </c>
       <c r="D112" t="str">
-        <v>Sentetik Monitör Model</v>
+        <v>Dell P2419H</v>
       </c>
       <c r="E112" t="str">
         <v>TKAJ-AJET A.Ş.</v>
@@ -2994,16 +2994,16 @@
     </row>
     <row r="113">
       <c r="A113" t="str">
-        <v>SYNPC000183</v>
+        <v>0CV8HSP</v>
       </c>
       <c r="B113" t="str">
-        <v>Kullanıcı 296</v>
+        <v>İbrahim Şahin</v>
       </c>
       <c r="C113" t="str">
         <v>EGITIM MERKEZI</v>
       </c>
       <c r="D113" t="str">
-        <v>Sentetik OptiPlex SYN</v>
+        <v>Lenovo ThinkCentre M90</v>
       </c>
       <c r="E113" t="str">
         <v>TKAJ-AJET A.Ş.</v>
@@ -3017,16 +3017,16 @@
     </row>
     <row r="114">
       <c r="A114" t="str">
-        <v>SYNPC000960</v>
+        <v>0AGQNGK</v>
       </c>
       <c r="B114" t="str">
-        <v>Kullanıcı 36</v>
+        <v>Ahmet Demir</v>
       </c>
       <c r="C114" t="str">
         <v>SUBE-C</v>
       </c>
       <c r="D114" t="str">
-        <v>Sentetik ThinkPad SYN</v>
+        <v>Lenovo ThinkPad X1 Carbon</v>
       </c>
       <c r="E114" t="str">
         <v>TKAO-THY A.O.</v>
@@ -3040,16 +3040,16 @@
     </row>
     <row r="115">
       <c r="A115" t="str">
-        <v>SYNPC000777</v>
+        <v>09Q7VNJ</v>
       </c>
       <c r="B115" t="str">
-        <v>Kullanıcı 285</v>
+        <v>Aslı Çelik</v>
       </c>
       <c r="C115" t="str">
         <v>DEPO-1</v>
       </c>
       <c r="D115" t="str">
-        <v>Sentetik OptiPlex SYN</v>
+        <v>Dell OptiPlex 5090</v>
       </c>
       <c r="E115" t="str">
         <v>TKAO-THY A.O.</v>
@@ -3063,16 +3063,16 @@
     </row>
     <row r="116">
       <c r="A116" t="str">
-        <v>SYNPC000012</v>
+        <v>PFJZ7J7T</v>
       </c>
       <c r="B116" t="str">
-        <v>Kullanıcı 211</v>
+        <v>Osman Yılmaz</v>
       </c>
       <c r="C116" t="str">
         <v>SUBE-B</v>
       </c>
       <c r="D116" t="str">
-        <v>Sentetik ThinkPad SYN</v>
+        <v>HP EliteBook 840 G8</v>
       </c>
       <c r="E116" t="str">
         <v>TKAO-THY A.O.</v>
@@ -3086,16 +3086,16 @@
     </row>
     <row r="117">
       <c r="A117" t="str">
-        <v>SYNPC001682</v>
+        <v>02541G3</v>
       </c>
       <c r="B117" t="str">
-        <v>Kullanıcı 170</v>
+        <v>Cem Yılmaz</v>
       </c>
       <c r="C117" t="str">
         <v>MERKEZ BINA</v>
       </c>
       <c r="D117" t="str">
-        <v>Sentetik ThinkPad SYN</v>
+        <v>Lenovo ThinkPad X1 Carbon</v>
       </c>
       <c r="E117" t="str">
         <v>TKAO-THY A.O.</v>
@@ -3109,16 +3109,16 @@
     </row>
     <row r="118">
       <c r="A118" t="str">
-        <v>SYNPC000554</v>
+        <v>0128X6R</v>
       </c>
       <c r="B118" t="str">
-        <v>Kullanıcı 3</v>
+        <v>Emine Demir</v>
       </c>
       <c r="C118" t="str">
         <v>MERKEZ BINA</v>
       </c>
       <c r="D118" t="str">
-        <v>Sentetik ThinkPad SYN</v>
+        <v>Dell Latitude 5420</v>
       </c>
       <c r="E118" t="str">
         <v>TKAO-THY A.O.</v>
@@ -3132,16 +3132,16 @@
     </row>
     <row r="119">
       <c r="A119" t="str">
-        <v>SYNPC000567</v>
+        <v>PFDZNR6H</v>
       </c>
       <c r="B119" t="str">
-        <v>Kullanıcı 258</v>
+        <v>Ozan Demir</v>
       </c>
       <c r="C119" t="str">
         <v>MERKEZ BINA</v>
       </c>
       <c r="D119" t="str">
-        <v>Sentetik ThinkPad SYN</v>
+        <v>HP EliteBook 840 G8</v>
       </c>
       <c r="E119" t="str">
         <v>TKAJ-AJET A.Ş.</v>
@@ -3155,16 +3155,16 @@
     </row>
     <row r="120">
       <c r="A120" t="str">
-        <v>SYNPC000117</v>
+        <v>PF6J8T57</v>
       </c>
       <c r="B120" t="str">
-        <v>Kullanıcı 217</v>
+        <v>Mustafa Demir</v>
       </c>
       <c r="C120" t="str">
         <v>LOJISTIK MERKEZI</v>
       </c>
       <c r="D120" t="str">
-        <v>Sentetik ThinkPad SYN</v>
+        <v>Lenovo ThinkPad T14</v>
       </c>
       <c r="E120" t="str">
         <v>TKAO-THY A.O.</v>
@@ -3178,16 +3178,16 @@
     </row>
     <row r="121">
       <c r="A121" t="str">
-        <v>SYNMN000107</v>
+        <v>CN0039A0L</v>
       </c>
       <c r="B121" t="str">
-        <v>Kullanıcı 145</v>
+        <v>Barış Çelik</v>
       </c>
       <c r="C121" t="str">
         <v>EGITIM MERKEZI</v>
       </c>
       <c r="D121" t="str">
-        <v>Sentetik Monitör Model</v>
+        <v>Samsung S24R350</v>
       </c>
       <c r="E121" t="str">
         <v>TKAJ-AJET A.Ş.</v>
@@ -3201,16 +3201,16 @@
     </row>
     <row r="122">
       <c r="A122" t="str">
-        <v>SYNPC001590</v>
+        <v>02XUG5U</v>
       </c>
       <c r="B122" t="str">
-        <v>Kullanıcı 89</v>
+        <v>Şeyma Yılmaz</v>
       </c>
       <c r="C122" t="str">
         <v>SUBE-C</v>
       </c>
       <c r="D122" t="str">
-        <v>Sentetik OptiPlex SYN</v>
+        <v>Lenovo ThinkCentre M90</v>
       </c>
       <c r="E122" t="str">
         <v>TKAO-THY A.O.</v>
@@ -3224,16 +3224,16 @@
     </row>
     <row r="123">
       <c r="A123" t="str">
-        <v>SYNMN000435</v>
+        <v>CN00D7A7E</v>
       </c>
       <c r="B123" t="str">
-        <v>Kullanıcı 233</v>
+        <v>Pınar Demir</v>
       </c>
       <c r="C123" t="str">
         <v>MERKEZ BINA</v>
       </c>
       <c r="D123" t="str">
-        <v>Sentetik Monitör Model</v>
+        <v>Samsung S24R350</v>
       </c>
       <c r="E123" t="str">
         <v>TKAJ-AJET A.Ş.</v>
@@ -3247,16 +3247,16 @@
     </row>
     <row r="124">
       <c r="A124" t="str">
-        <v>SYNMN000542</v>
+        <v>CN00GFK6R</v>
       </c>
       <c r="B124" t="str">
-        <v>Kullanıcı 188</v>
+        <v>Gizem Yıldırım</v>
       </c>
       <c r="C124" t="str">
         <v>MERKEZ BINA</v>
       </c>
       <c r="D124" t="str">
-        <v>Sentetik Monitör Model</v>
+        <v>LG 24MK430H</v>
       </c>
       <c r="E124" t="str">
         <v>TKAO-THY A.O.</v>
@@ -3270,16 +3270,16 @@
     </row>
     <row r="125">
       <c r="A125" t="str">
-        <v>SYNPC000160</v>
+        <v>0JHFFHL</v>
       </c>
       <c r="B125" t="str">
-        <v>Kullanıcı 288</v>
+        <v>Şeyma Demir</v>
       </c>
       <c r="C125" t="str">
         <v>SAHA OFISI-1</v>
       </c>
       <c r="D125" t="str">
-        <v>Sentetik OptiPlex SYN</v>
+        <v>Dell OptiPlex 7090</v>
       </c>
       <c r="E125" t="str">
         <v>TKAJ-AJET A.Ş.</v>
@@ -3293,16 +3293,16 @@
     </row>
     <row r="126">
       <c r="A126" t="str">
-        <v>SYNPC001050</v>
+        <v>0D8KCVA</v>
       </c>
       <c r="B126" t="str">
-        <v>Kullanıcı 272</v>
+        <v>Aslı Şahin</v>
       </c>
       <c r="C126" t="str">
         <v>SAHA OFISI-2</v>
       </c>
       <c r="D126" t="str">
-        <v>Sentetik OptiPlex SYN</v>
+        <v>Lenovo ThinkCentre M90</v>
       </c>
       <c r="E126" t="str">
         <v>TKAJ-AJET A.Ş.</v>
@@ -3316,16 +3316,16 @@
     </row>
     <row r="127">
       <c r="A127" t="str">
-        <v>SYNPC001307</v>
+        <v>0L9ZSAW</v>
       </c>
       <c r="B127" t="str">
-        <v>Kullanıcı 124</v>
+        <v>Ahmet Doğan</v>
       </c>
       <c r="C127" t="str">
         <v>SAHA OFISI-1</v>
       </c>
       <c r="D127" t="str">
-        <v>Sentetik OptiPlex SYN</v>
+        <v>Dell OptiPlex 7090</v>
       </c>
       <c r="E127" t="str">
         <v>TKAJ-AJET A.Ş.</v>
@@ -3339,16 +3339,16 @@
     </row>
     <row r="128">
       <c r="A128" t="str">
-        <v>SYNPC001045</v>
+        <v>09ZMEUB</v>
       </c>
       <c r="B128" t="str">
-        <v>Kullanıcı 150</v>
+        <v>Meryem Kaya</v>
       </c>
       <c r="C128" t="str">
         <v>DEPO-1</v>
       </c>
       <c r="D128" t="str">
-        <v>Sentetik OptiPlex SYN</v>
+        <v>Lenovo ThinkCentre M90</v>
       </c>
       <c r="E128" t="str">
         <v>TKAJ-AJET A.Ş.</v>
@@ -3362,16 +3362,16 @@
     </row>
     <row r="129">
       <c r="A129" t="str">
-        <v>SYNMN000400</v>
+        <v>CN00C57X5</v>
       </c>
       <c r="B129" t="str">
-        <v>Kullanıcı 171</v>
+        <v>Hasan Öztürk</v>
       </c>
       <c r="C129" t="str">
         <v>EGITIM MERKEZI</v>
       </c>
       <c r="D129" t="str">
-        <v>Sentetik Monitör Model</v>
+        <v>Dell P2419H</v>
       </c>
       <c r="E129" t="str">
         <v>TKAJ-AJET A.Ş.</v>
@@ -3385,16 +3385,16 @@
     </row>
     <row r="130">
       <c r="A130" t="str">
-        <v>SYNPC000615</v>
+        <v>PF63CPUQ</v>
       </c>
       <c r="B130" t="str">
-        <v>Kullanıcı 87</v>
+        <v>Onur Yıldız</v>
       </c>
       <c r="C130" t="str">
         <v>SAHA OFISI-1</v>
       </c>
       <c r="D130" t="str">
-        <v>Sentetik ThinkPad SYN</v>
+        <v>Dell Latitude 5420</v>
       </c>
       <c r="E130" t="str">
         <v>TKAJ-AJET A.Ş.</v>
@@ -3408,16 +3408,16 @@
     </row>
     <row r="131">
       <c r="A131" t="str">
-        <v>SYNPC000413</v>
+        <v>06TH33F</v>
       </c>
       <c r="B131" t="str">
-        <v>Kullanıcı 194</v>
+        <v>Mehmet Yıldırım</v>
       </c>
       <c r="C131" t="str">
         <v>SUBE-C</v>
       </c>
       <c r="D131" t="str">
-        <v>Sentetik OptiPlex SYN</v>
+        <v>HP EliteDesk 800 G6</v>
       </c>
       <c r="E131" t="str">
         <v>TKAO-THY A.O.</v>
@@ -3431,16 +3431,16 @@
     </row>
     <row r="132">
       <c r="A132" t="str">
-        <v>SYNMN000598</v>
+        <v>CN00J599K</v>
       </c>
       <c r="B132" t="str">
-        <v>Kullanıcı 315</v>
+        <v>Büşra Kaya</v>
       </c>
       <c r="C132" t="str">
         <v>SAHA OFISI-2</v>
       </c>
       <c r="D132" t="str">
-        <v>Sentetik Monitör Model</v>
+        <v>LG 24MK430H</v>
       </c>
       <c r="E132" t="str">
         <v>TKAJ-AJET A.Ş.</v>
@@ -3454,16 +3454,16 @@
     </row>
     <row r="133">
       <c r="A133" t="str">
-        <v>SYNPC000237</v>
+        <v>095ERAY</v>
       </c>
       <c r="B133" t="str">
-        <v>Kullanıcı 36</v>
+        <v>Ahmet Demir</v>
       </c>
       <c r="C133" t="str">
         <v>DEPO-1</v>
       </c>
       <c r="D133" t="str">
-        <v>Sentetik OptiPlex SYN</v>
+        <v>Dell OptiPlex 7090</v>
       </c>
       <c r="E133" t="str">
         <v>TKAO-THY A.O.</v>
@@ -3477,16 +3477,16 @@
     </row>
     <row r="134">
       <c r="A134" t="str">
-        <v>SYNMN000179</v>
+        <v>CN005FGPN</v>
       </c>
       <c r="B134" t="str">
-        <v>Kullanıcı 283</v>
+        <v>Meryem Yılmaz</v>
       </c>
       <c r="C134" t="str">
         <v>SUBE-C</v>
       </c>
       <c r="D134" t="str">
-        <v>Sentetik Monitör Model</v>
+        <v>Samsung S24R350</v>
       </c>
       <c r="E134" t="str">
         <v>TKAO-THY A.O.</v>
@@ -3500,16 +3500,16 @@
     </row>
     <row r="135">
       <c r="A135" t="str">
-        <v>SYNPC001588</v>
+        <v>0DSZXZZ</v>
       </c>
       <c r="B135" t="str">
-        <v>Kullanıcı 229</v>
+        <v>Ahmet Aslan</v>
       </c>
       <c r="C135" t="str">
         <v>LOJISTIK MERKEZI</v>
       </c>
       <c r="D135" t="str">
-        <v>Sentetik ThinkPad SYN</v>
+        <v>Lenovo ThinkPad T14</v>
       </c>
       <c r="E135" t="str">
         <v>TKAJ-AJET A.Ş.</v>
@@ -3523,16 +3523,16 @@
     </row>
     <row r="136">
       <c r="A136" t="str">
-        <v>SYNPC001579</v>
+        <v>PFUWPV7X</v>
       </c>
       <c r="B136" t="str">
-        <v>Kullanıcı 117</v>
+        <v>Ahmet Yılmaz</v>
       </c>
       <c r="C136" t="str">
         <v>MERKEZ BINA</v>
       </c>
       <c r="D136" t="str">
-        <v>Sentetik ThinkPad SYN</v>
+        <v>HP EliteBook 840 G8</v>
       </c>
       <c r="E136" t="str">
         <v>TKAO-THY A.O.</v>
@@ -3546,16 +3546,16 @@
     </row>
     <row r="137">
       <c r="A137" t="str">
-        <v>SYNPC000681</v>
+        <v>009S4CQ</v>
       </c>
       <c r="B137" t="str">
-        <v>Kullanıcı 238</v>
+        <v>Murat Demir</v>
       </c>
       <c r="C137" t="str">
         <v>SUBE-C</v>
       </c>
       <c r="D137" t="str">
-        <v>Sentetik OptiPlex SYN</v>
+        <v>Dell OptiPlex 5090</v>
       </c>
       <c r="E137" t="str">
         <v>TKAJ-AJET A.Ş.</v>
@@ -3569,16 +3569,16 @@
     </row>
     <row r="138">
       <c r="A138" t="str">
-        <v>SYNPC001793</v>
+        <v>PF1GHTVK</v>
       </c>
       <c r="B138" t="str">
-        <v>Kullanıcı 124</v>
+        <v>Ahmet Doğan</v>
       </c>
       <c r="C138" t="str">
         <v>SAHA OFISI-2</v>
       </c>
       <c r="D138" t="str">
-        <v>Sentetik ThinkPad SYN</v>
+        <v>HP EliteBook 840 G8</v>
       </c>
       <c r="E138" t="str">
         <v>TKAJ-AJET A.Ş.</v>
@@ -3592,16 +3592,16 @@
     </row>
     <row r="139">
       <c r="A139" t="str">
-        <v>SYNPC000045</v>
+        <v>01B9X5M</v>
       </c>
       <c r="B139" t="str">
-        <v>Kullanıcı 42</v>
+        <v>Merve Çelik</v>
       </c>
       <c r="C139" t="str">
         <v>SAHA OFISI-2</v>
       </c>
       <c r="D139" t="str">
-        <v>Sentetik ThinkPad SYN</v>
+        <v>Dell Latitude 5420</v>
       </c>
       <c r="E139" t="str">
         <v>TKAO-THY A.O.</v>
@@ -3615,16 +3615,16 @@
     </row>
     <row r="140">
       <c r="A140" t="str">
-        <v>SYNPC001502</v>
+        <v>PF4KTRE3</v>
       </c>
       <c r="B140" t="str">
-        <v>Kullanıcı 82</v>
+        <v>Mustafa Çelik</v>
       </c>
       <c r="C140" t="str">
         <v>EGITIM MERKEZI</v>
       </c>
       <c r="D140" t="str">
-        <v>Sentetik ThinkPad SYN</v>
+        <v>Lenovo ThinkPad X1 Carbon</v>
       </c>
       <c r="E140" t="str">
         <v>TKAJ-AJET A.Ş.</v>
@@ -3638,16 +3638,16 @@
     </row>
     <row r="141">
       <c r="A141" t="str">
-        <v>SYNPC001153</v>
+        <v>PFP1GHFU</v>
       </c>
       <c r="B141" t="str">
-        <v>Kullanıcı 88</v>
+        <v>Büşra Öztürk</v>
       </c>
       <c r="C141" t="str">
         <v>SAHA OFISI-2</v>
       </c>
       <c r="D141" t="str">
-        <v>Sentetik ThinkPad SYN</v>
+        <v>Dell Latitude 5420</v>
       </c>
       <c r="E141" t="str">
         <v>TKAJ-AJET A.Ş.</v>
@@ -3661,16 +3661,16 @@
     </row>
     <row r="142">
       <c r="A142" t="str">
-        <v>SYNPC001395</v>
+        <v>0FVWL8L</v>
       </c>
       <c r="B142" t="str">
-        <v>Kullanıcı 186</v>
+        <v>Derya Demir</v>
       </c>
       <c r="C142" t="str">
         <v>SUBE-A</v>
       </c>
       <c r="D142" t="str">
-        <v>Sentetik OptiPlex SYN</v>
+        <v>Dell OptiPlex 5090</v>
       </c>
       <c r="E142" t="str">
         <v>TKAJ-AJET A.Ş.</v>
@@ -3684,16 +3684,16 @@
     </row>
     <row r="143">
       <c r="A143" t="str">
-        <v>SYNMN000417</v>
+        <v>CN00CNRJN</v>
       </c>
       <c r="B143" t="str">
-        <v>Kullanıcı 119</v>
+        <v>Meryem Yıldırım</v>
       </c>
       <c r="C143" t="str">
         <v>DEPO-1</v>
       </c>
       <c r="D143" t="str">
-        <v>Sentetik Monitör Model</v>
+        <v>Dell U2419H</v>
       </c>
       <c r="E143" t="str">
         <v>TKAO-THY A.O.</v>
@@ -3707,16 +3707,16 @@
     </row>
     <row r="144">
       <c r="A144" t="str">
-        <v>SYNMN000496</v>
+        <v>CN00F25GK</v>
       </c>
       <c r="B144" t="str">
-        <v>Kullanıcı 259</v>
+        <v>Aslı Yılmaz</v>
       </c>
       <c r="C144" t="str">
         <v>EGITIM MERKEZI</v>
       </c>
       <c r="D144" t="str">
-        <v>Sentetik Monitör Model</v>
+        <v>Dell P2419H</v>
       </c>
       <c r="E144" t="str">
         <v>TKAJ-AJET A.Ş.</v>
@@ -3730,16 +3730,16 @@
     </row>
     <row r="145">
       <c r="A145" t="str">
-        <v>SYNMN000791</v>
+        <v>CN00Q05FN</v>
       </c>
       <c r="B145" t="str">
-        <v>Kullanıcı 7</v>
+        <v>Elif Yılmaz</v>
       </c>
       <c r="C145" t="str">
         <v>EGITIM MERKEZI</v>
       </c>
       <c r="D145" t="str">
-        <v>Sentetik Monitör Model</v>
+        <v>Samsung S24R350</v>
       </c>
       <c r="E145" t="str">
         <v>TKAJ-AJET A.Ş.</v>
@@ -3753,16 +3753,16 @@
     </row>
     <row r="146">
       <c r="A146" t="str">
-        <v>SYNPC001680</v>
+        <v>PFYP3UJR</v>
       </c>
       <c r="B146" t="str">
-        <v>Kullanıcı 190</v>
+        <v>Şeyma Çelik</v>
       </c>
       <c r="C146" t="str">
         <v>SAHA OFISI-2</v>
       </c>
       <c r="D146" t="str">
-        <v>Sentetik ThinkPad SYN</v>
+        <v>HP EliteBook 840 G8</v>
       </c>
       <c r="E146" t="str">
         <v>TKAJ-AJET A.Ş.</v>
@@ -3776,16 +3776,16 @@
     </row>
     <row r="147">
       <c r="A147" t="str">
-        <v>SYNPC000809</v>
+        <v>0HRUQEL</v>
       </c>
       <c r="B147" t="str">
-        <v>Kullanıcı 287</v>
+        <v>Hatice Yılmaz</v>
       </c>
       <c r="C147" t="str">
         <v>SUBE-B</v>
       </c>
       <c r="D147" t="str">
-        <v>Sentetik ThinkPad SYN</v>
+        <v>HP EliteBook 840 G8</v>
       </c>
       <c r="E147" t="str">
         <v>TKAJ-AJET A.Ş.</v>
@@ -3799,16 +3799,16 @@
     </row>
     <row r="148">
       <c r="A148" t="str">
-        <v>SYNMN000709</v>
+        <v>CN00MHNDY</v>
       </c>
       <c r="B148" t="str">
-        <v>Kullanıcı 147</v>
+        <v>Onur Kaya</v>
       </c>
       <c r="C148" t="str">
         <v>SUBE-C</v>
       </c>
       <c r="D148" t="str">
-        <v>Sentetik Monitör Model</v>
+        <v>Dell U2419H</v>
       </c>
       <c r="E148" t="str">
         <v>TKAJ-AJET A.Ş.</v>
@@ -3822,16 +3822,16 @@
     </row>
     <row r="149">
       <c r="A149" t="str">
-        <v>SYNPC000519</v>
+        <v>07TX69M</v>
       </c>
       <c r="B149" t="str">
-        <v>Kullanıcı 225</v>
+        <v>Şeyma Yıldırım</v>
       </c>
       <c r="C149" t="str">
         <v>EGITIM MERKEZI</v>
       </c>
       <c r="D149" t="str">
-        <v>Sentetik OptiPlex SYN</v>
+        <v>Dell OptiPlex 7090</v>
       </c>
       <c r="E149" t="str">
         <v>TKAJ-AJET A.Ş.</v>
@@ -3845,16 +3845,16 @@
     </row>
     <row r="150">
       <c r="A150" t="str">
-        <v>SYNPC001437</v>
+        <v>06NDD1D</v>
       </c>
       <c r="B150" t="str">
-        <v>Kullanıcı 5</v>
+        <v>Nazlı Yılmaz</v>
       </c>
       <c r="C150" t="str">
         <v>MERKEZ BINA</v>
       </c>
       <c r="D150" t="str">
-        <v>Sentetik OptiPlex SYN</v>
+        <v>Lenovo ThinkCentre M90</v>
       </c>
       <c r="E150" t="str">
         <v>TKAO-THY A.O.</v>
@@ -3868,16 +3868,16 @@
     </row>
     <row r="151">
       <c r="A151" t="str">
-        <v>SYNMN000497</v>
+        <v>CN00F36HU</v>
       </c>
       <c r="B151" t="str">
-        <v>Kullanıcı 303</v>
+        <v>Serkan Yıldırım</v>
       </c>
       <c r="C151" t="str">
         <v>SUBE-B</v>
       </c>
       <c r="D151" t="str">
-        <v>Sentetik Monitör Model</v>
+        <v>Dell U2419H</v>
       </c>
       <c r="E151" t="str">
         <v>TKAJ-AJET A.Ş.</v>
@@ -3891,16 +3891,16 @@
     </row>
     <row r="152">
       <c r="A152" t="str">
-        <v>SYNPC000103</v>
+        <v>PFZUZVW7</v>
       </c>
       <c r="B152" t="str">
-        <v>Kullanıcı 219</v>
+        <v>Pınar Kaya</v>
       </c>
       <c r="C152" t="str">
         <v>MERKEZ BINA</v>
       </c>
       <c r="D152" t="str">
-        <v>Sentetik ThinkPad SYN</v>
+        <v>HP EliteBook 840 G8</v>
       </c>
       <c r="E152" t="str">
         <v>TKAJ-AJET A.Ş.</v>
@@ -3914,16 +3914,16 @@
     </row>
     <row r="153">
       <c r="A153" t="str">
-        <v>SYNMN000685</v>
+        <v>CN00LSXHL</v>
       </c>
       <c r="B153" t="str">
-        <v>Kullanıcı 72</v>
+        <v>İpek Demir</v>
       </c>
       <c r="C153" t="str">
         <v>SAHA OFISI-1</v>
       </c>
       <c r="D153" t="str">
-        <v>Sentetik Monitör Model</v>
+        <v>Dell U2419H</v>
       </c>
       <c r="E153" t="str">
         <v>TKAO-THY A.O.</v>
@@ -3937,16 +3937,16 @@
     </row>
     <row r="154">
       <c r="A154" t="str">
-        <v>SYNPC000838</v>
+        <v>0JT7KWA</v>
       </c>
       <c r="B154" t="str">
-        <v>Kullanıcı 160</v>
+        <v>Cem Demir</v>
       </c>
       <c r="C154" t="str">
         <v>SUBE-C</v>
       </c>
       <c r="D154" t="str">
-        <v>Sentetik OptiPlex SYN</v>
+        <v>Lenovo ThinkCentre M90</v>
       </c>
       <c r="E154" t="str">
         <v>TKAO-THY A.O.</v>
@@ -3960,16 +3960,16 @@
     </row>
     <row r="155">
       <c r="A155" t="str">
-        <v>SYNMN000078</v>
+        <v>CN002DDXX</v>
       </c>
       <c r="B155" t="str">
-        <v>Kullanıcı 308</v>
+        <v>Fatma Aydın</v>
       </c>
       <c r="C155" t="str">
         <v>SUBE-B</v>
       </c>
       <c r="D155" t="str">
-        <v>Sentetik Monitör Model</v>
+        <v>LG 24MK430H</v>
       </c>
       <c r="E155" t="str">
         <v>TKAO-THY A.O.</v>
@@ -3983,16 +3983,16 @@
     </row>
     <row r="156">
       <c r="A156" t="str">
-        <v>SYNPC000046</v>
+        <v>0FR0J28</v>
       </c>
       <c r="B156" t="str">
-        <v>Kullanıcı 261</v>
+        <v>Elif Aydın</v>
       </c>
       <c r="C156" t="str">
         <v>SUBE-C</v>
       </c>
       <c r="D156" t="str">
-        <v>Sentetik OptiPlex SYN</v>
+        <v>Dell OptiPlex 7090</v>
       </c>
       <c r="E156" t="str">
         <v>TKAO-THY A.O.</v>
@@ -4006,16 +4006,16 @@
     </row>
     <row r="157">
       <c r="A157" t="str">
-        <v>SYNPC000511</v>
+        <v>PFZBHN2A</v>
       </c>
       <c r="B157" t="str">
-        <v>Kullanıcı 109</v>
+        <v>Nazlı Yıldırım</v>
       </c>
       <c r="C157" t="str">
         <v>SAHA OFISI-1</v>
       </c>
       <c r="D157" t="str">
-        <v>Sentetik ThinkPad SYN</v>
+        <v>Dell Latitude 5420</v>
       </c>
       <c r="E157" t="str">
         <v>TKAJ-AJET A.Ş.</v>
@@ -4029,16 +4029,16 @@
     </row>
     <row r="158">
       <c r="A158" t="str">
-        <v>SYNPC001702</v>
+        <v>PFLMRF55</v>
       </c>
       <c r="B158" t="str">
-        <v>Kullanıcı 204</v>
+        <v>Ebru Yıldırım</v>
       </c>
       <c r="C158" t="str">
         <v>LOJISTIK MERKEZI</v>
       </c>
       <c r="D158" t="str">
-        <v>Sentetik ThinkPad SYN</v>
+        <v>HP EliteBook 840 G8</v>
       </c>
       <c r="E158" t="str">
         <v>TKAJ-AJET A.Ş.</v>
@@ -4052,16 +4052,16 @@
     </row>
     <row r="159">
       <c r="A159" t="str">
-        <v>SYNMN000656</v>
+        <v>CN00KX1EX</v>
       </c>
       <c r="B159" t="str">
-        <v>Kullanıcı 206</v>
+        <v>Gizem Yılmaz</v>
       </c>
       <c r="C159" t="str">
         <v>EGITIM MERKEZI</v>
       </c>
       <c r="D159" t="str">
-        <v>Sentetik Monitör Model</v>
+        <v>Dell P2419H</v>
       </c>
       <c r="E159" t="str">
         <v>TKAO-THY A.O.</v>
@@ -4075,16 +4075,16 @@
     </row>
     <row r="160">
       <c r="A160" t="str">
-        <v>SYNPC001962</v>
+        <v>0CMPSMF</v>
       </c>
       <c r="B160" t="str">
-        <v>Kullanıcı 125</v>
+        <v>Mustafa Kaya</v>
       </c>
       <c r="C160" t="str">
         <v>MERKEZ BINA</v>
       </c>
       <c r="D160" t="str">
-        <v>Sentetik OptiPlex SYN</v>
+        <v>Lenovo ThinkCentre M90</v>
       </c>
       <c r="E160" t="str">
         <v>TKAO-THY A.O.</v>
@@ -4098,16 +4098,16 @@
     </row>
     <row r="161">
       <c r="A161" t="str">
-        <v>SYNPC000391</v>
+        <v>0CFQ0UC</v>
       </c>
       <c r="B161" t="str">
-        <v>Kullanıcı 289</v>
+        <v>Gizem Yıldız</v>
       </c>
       <c r="C161" t="str">
         <v>MERKEZ BINA</v>
       </c>
       <c r="D161" t="str">
-        <v>Sentetik OptiPlex SYN</v>
+        <v>HP EliteDesk 800 G6</v>
       </c>
       <c r="E161" t="str">
         <v>TKAO-THY A.O.</v>
@@ -4121,16 +4121,16 @@
     </row>
     <row r="162">
       <c r="A162" t="str">
-        <v>SYNPC000848</v>
+        <v>01R6ZAV</v>
       </c>
       <c r="B162" t="str">
-        <v>Kullanıcı 278</v>
+        <v>Barış Kaya</v>
       </c>
       <c r="C162" t="str">
-        <v>GENEL MUDURLUK (SENTETIK)</v>
+        <v>GENEL MUDURLUK</v>
       </c>
       <c r="D162" t="str">
-        <v>Sentetik ThinkPad SYN</v>
+        <v>Lenovo ThinkPad X1 Carbon</v>
       </c>
       <c r="E162" t="str">
         <v>TKAO-THY A.O.</v>
@@ -4144,16 +4144,16 @@
     </row>
     <row r="163">
       <c r="A163" t="str">
-        <v>SYNPC001761</v>
+        <v>PF09XJ9C</v>
       </c>
       <c r="B163" t="str">
-        <v>Kullanıcı 286</v>
+        <v>Derya Özdemir</v>
       </c>
       <c r="C163" t="str">
-        <v>GENEL MUDURLUK (SENTETIK)</v>
+        <v>GENEL MUDURLUK</v>
       </c>
       <c r="D163" t="str">
-        <v>Sentetik ThinkPad SYN</v>
+        <v>Lenovo ThinkPad T14</v>
       </c>
       <c r="E163" t="str">
         <v>TKAO-THY A.O.</v>
@@ -4167,16 +4167,16 @@
     </row>
     <row r="164">
       <c r="A164" t="str">
-        <v>SYNPC001567</v>
+        <v>07SKUT6</v>
       </c>
       <c r="B164" t="str">
-        <v>Kullanıcı 294</v>
+        <v>Cem Yıldırım</v>
       </c>
       <c r="C164" t="str">
         <v>MERKEZ BINA</v>
       </c>
       <c r="D164" t="str">
-        <v>Sentetik OptiPlex SYN</v>
+        <v>Lenovo ThinkCentre M90</v>
       </c>
       <c r="E164" t="str">
         <v>TKAO-THY A.O.</v>
@@ -4190,16 +4190,16 @@
     </row>
     <row r="165">
       <c r="A165" t="str">
-        <v>SYNPC000002</v>
+        <v>06T4HWJ</v>
       </c>
       <c r="B165" t="str">
-        <v>Kullanıcı 69</v>
+        <v>Mehmet Yılmaz</v>
       </c>
       <c r="C165" t="str">
         <v>SAHA OFISI-2</v>
       </c>
       <c r="D165" t="str">
-        <v>Sentetik OptiPlex SYN</v>
+        <v>Dell OptiPlex 5090</v>
       </c>
       <c r="E165" t="str">
         <v>TKAJ-AJET A.Ş.</v>
@@ -4213,16 +4213,16 @@
     </row>
     <row r="166">
       <c r="A166" t="str">
-        <v>SYNMN000779</v>
+        <v>CN00PMT0G</v>
       </c>
       <c r="B166" t="str">
-        <v>Kullanıcı 202</v>
+        <v>Mehmet Kaya</v>
       </c>
       <c r="C166" t="str">
         <v>SUBE-B</v>
       </c>
       <c r="D166" t="str">
-        <v>Sentetik Monitör Model</v>
+        <v>Samsung S24R350</v>
       </c>
       <c r="E166" t="str">
         <v>TKAJ-AJET A.Ş.</v>
@@ -4236,16 +4236,16 @@
     </row>
     <row r="167">
       <c r="A167" t="str">
-        <v>SYNPC000013</v>
+        <v>0KKY0L1</v>
       </c>
       <c r="B167" t="str">
-        <v>Kullanıcı 224</v>
+        <v>Yusuf Yılmaz</v>
       </c>
       <c r="C167" t="str">
         <v>SAHA OFISI-1</v>
       </c>
       <c r="D167" t="str">
-        <v>Sentetik OptiPlex SYN</v>
+        <v>Dell OptiPlex 7090</v>
       </c>
       <c r="E167" t="str">
         <v>TKAJ-AJET A.Ş.</v>
@@ -4259,16 +4259,16 @@
     </row>
     <row r="168">
       <c r="A168" t="str">
-        <v>SYNMN000278</v>
+        <v>CN008FHCV</v>
       </c>
       <c r="B168" t="str">
-        <v>Kullanıcı 116</v>
+        <v>Gizem Çelik</v>
       </c>
       <c r="C168" t="str">
         <v>EGITIM MERKEZI</v>
       </c>
       <c r="D168" t="str">
-        <v>Sentetik Monitör Model</v>
+        <v>LG 24MK430H</v>
       </c>
       <c r="E168" t="str">
         <v>TKAJ-AJET A.Ş.</v>
@@ -4282,16 +4282,16 @@
     </row>
     <row r="169">
       <c r="A169" t="str">
-        <v>SYNPC000308</v>
+        <v>087FP7Y</v>
       </c>
       <c r="B169" t="str">
-        <v>Kullanıcı 32</v>
+        <v>İbrahim Yılmaz</v>
       </c>
       <c r="C169" t="str">
         <v>SUBE-C</v>
       </c>
       <c r="D169" t="str">
-        <v>Sentetik OptiPlex SYN</v>
+        <v>Dell OptiPlex 5090</v>
       </c>
       <c r="E169" t="str">
         <v>TKAJ-AJET A.Ş.</v>
@@ -4305,16 +4305,16 @@
     </row>
     <row r="170">
       <c r="A170" t="str">
-        <v>SYNPC000886</v>
+        <v>PFQJJWR6</v>
       </c>
       <c r="B170" t="str">
-        <v>Kullanıcı 34</v>
+        <v>İbrahim Demir</v>
       </c>
       <c r="C170" t="str">
-        <v>GENEL MUDURLUK (SENTETIK)</v>
+        <v>GENEL MUDURLUK</v>
       </c>
       <c r="D170" t="str">
-        <v>Sentetik ThinkPad SYN</v>
+        <v>Dell Latitude 5420</v>
       </c>
       <c r="E170" t="str">
         <v>TKAO-THY A.O.</v>
@@ -4328,16 +4328,16 @@
     </row>
     <row r="171">
       <c r="A171" t="str">
-        <v>SYNPC001860</v>
+        <v>0CER8JU</v>
       </c>
       <c r="B171" t="str">
-        <v>Kullanıcı 250</v>
+        <v>Selin Özdemir</v>
       </c>
       <c r="C171" t="str">
-        <v>GENEL MUDURLUK (SENTETIK)</v>
+        <v>GENEL MUDURLUK</v>
       </c>
       <c r="D171" t="str">
-        <v>Sentetik OptiPlex SYN</v>
+        <v>Dell OptiPlex 5090</v>
       </c>
       <c r="E171" t="str">
         <v>TKAO-THY A.O.</v>
@@ -4351,16 +4351,16 @@
     </row>
     <row r="172">
       <c r="A172" t="str">
-        <v>SYNPC001293</v>
+        <v>0943DUH</v>
       </c>
       <c r="B172" t="str">
-        <v>Kullanıcı 26</v>
+        <v>Burak Çetin</v>
       </c>
       <c r="C172" t="str">
         <v>MERKEZ BINA</v>
       </c>
       <c r="D172" t="str">
-        <v>Sentetik OptiPlex SYN</v>
+        <v>Dell OptiPlex 7090</v>
       </c>
       <c r="E172" t="str">
         <v>TKAO-THY A.O.</v>
@@ -4374,16 +4374,16 @@
     </row>
     <row r="173">
       <c r="A173" t="str">
-        <v>SYNMN000403</v>
+        <v>CN00C8B0Y</v>
       </c>
       <c r="B173" t="str">
-        <v>Kullanıcı 309</v>
+        <v>Kemal Yılmaz</v>
       </c>
       <c r="C173" t="str">
         <v>DEPO-1</v>
       </c>
       <c r="D173" t="str">
-        <v>Sentetik Monitör Model</v>
+        <v>Samsung S24R350</v>
       </c>
       <c r="E173" t="str">
         <v>TKAJ-AJET A.Ş.</v>
@@ -4397,16 +4397,16 @@
     </row>
     <row r="174">
       <c r="A174" t="str">
-        <v>SYNPC001644</v>
+        <v>03S15P7</v>
       </c>
       <c r="B174" t="str">
-        <v>Kullanıcı 31</v>
+        <v>Serkan Çelik</v>
       </c>
       <c r="C174" t="str">
         <v>DEPO-1</v>
       </c>
       <c r="D174" t="str">
-        <v>Sentetik OptiPlex SYN</v>
+        <v>Dell OptiPlex 5090</v>
       </c>
       <c r="E174" t="str">
         <v>TKAO-THY A.O.</v>
@@ -4420,16 +4420,16 @@
     </row>
     <row r="175">
       <c r="A175" t="str">
-        <v>SYNPC000338</v>
+        <v>076FCZ5</v>
       </c>
       <c r="B175" t="str">
-        <v>Kullanıcı 157</v>
+        <v>Nazlı Çelik</v>
       </c>
       <c r="C175" t="str">
         <v>EGITIM MERKEZI</v>
       </c>
       <c r="D175" t="str">
-        <v>Sentetik ThinkPad SYN</v>
+        <v>HP EliteBook 840 G8</v>
       </c>
       <c r="E175" t="str">
         <v>TKAO-THY A.O.</v>
@@ -4443,16 +4443,16 @@
     </row>
     <row r="176">
       <c r="A176" t="str">
-        <v>SYNPC001073</v>
+        <v>04BEH3E</v>
       </c>
       <c r="B176" t="str">
-        <v>Kullanıcı 222</v>
+        <v>Büşra Demir</v>
       </c>
       <c r="C176" t="str">
         <v>SUBE-A</v>
       </c>
       <c r="D176" t="str">
-        <v>Sentetik OptiPlex SYN</v>
+        <v>Dell OptiPlex 7090</v>
       </c>
       <c r="E176" t="str">
         <v>TKAO-THY A.O.</v>
@@ -4466,16 +4466,16 @@
     </row>
     <row r="177">
       <c r="A177" t="str">
-        <v>SYNPC000463</v>
+        <v>PFSEMG83</v>
       </c>
       <c r="B177" t="str">
-        <v>Kullanıcı 86</v>
+        <v>Merve Yılmaz</v>
       </c>
       <c r="C177" t="str">
         <v>EGITIM MERKEZI</v>
       </c>
       <c r="D177" t="str">
-        <v>Sentetik ThinkPad SYN</v>
+        <v>Dell Latitude 5420</v>
       </c>
       <c r="E177" t="str">
         <v>TKAJ-AJET A.Ş.</v>
@@ -4489,16 +4489,16 @@
     </row>
     <row r="178">
       <c r="A178" t="str">
-        <v>SYNPC001794</v>
+        <v>03BRJB2</v>
       </c>
       <c r="B178" t="str">
-        <v>Kullanıcı 317</v>
+        <v>Onur Demir</v>
       </c>
       <c r="C178" t="str">
         <v>SAHA OFISI-2</v>
       </c>
       <c r="D178" t="str">
-        <v>Sentetik OptiPlex SYN</v>
+        <v>Lenovo ThinkCentre M90</v>
       </c>
       <c r="E178" t="str">
         <v>TKAO-THY A.O.</v>
@@ -4512,16 +4512,16 @@
     </row>
     <row r="179">
       <c r="A179" t="str">
-        <v>SYNMN000686</v>
+        <v>CN00LTYJV</v>
       </c>
       <c r="B179" t="str">
-        <v>Kullanıcı 135</v>
+        <v>Barış Demir</v>
       </c>
       <c r="C179" t="str">
         <v>DEPO-1</v>
       </c>
       <c r="D179" t="str">
-        <v>Sentetik Monitör Model</v>
+        <v>LG 24MK430H</v>
       </c>
       <c r="E179" t="str">
         <v>TKAJ-AJET A.Ş.</v>
@@ -4535,16 +4535,16 @@
     </row>
     <row r="180">
       <c r="A180" t="str">
-        <v>SYNMN000168</v>
+        <v>CN005459R</v>
       </c>
       <c r="B180" t="str">
-        <v>Kullanıcı 151</v>
+        <v>Ali Özdemir</v>
       </c>
       <c r="C180" t="str">
         <v>LOJISTIK MERKEZI</v>
       </c>
       <c r="D180" t="str">
-        <v>Sentetik Monitör Model</v>
+        <v>Dell P2419H</v>
       </c>
       <c r="E180" t="str">
         <v>TKAJ-AJET A.Ş.</v>
@@ -4558,16 +4558,16 @@
     </row>
     <row r="181">
       <c r="A181" t="str">
-        <v>SYNMN000559</v>
+        <v>CN00GZ2U8</v>
       </c>
       <c r="B181" t="str">
-        <v>Kullanıcı 157</v>
+        <v>Nazlı Çelik</v>
       </c>
       <c r="C181" t="str">
         <v>EGITIM MERKEZI</v>
       </c>
       <c r="D181" t="str">
-        <v>Sentetik Monitör Model</v>
+        <v>Samsung S24R350</v>
       </c>
       <c r="E181" t="str">
         <v>TKAO-THY A.O.</v>
@@ -4581,16 +4581,16 @@
     </row>
     <row r="182">
       <c r="A182" t="str">
-        <v>SYNPC000931</v>
+        <v>0C71L2D</v>
       </c>
       <c r="B182" t="str">
-        <v>Kullanıcı 1</v>
+        <v>Hüseyin Özdemir</v>
       </c>
       <c r="C182" t="str">
         <v>DEPO-1</v>
       </c>
       <c r="D182" t="str">
-        <v>Sentetik OptiPlex SYN</v>
+        <v>Dell OptiPlex 5090</v>
       </c>
       <c r="E182" t="str">
         <v>TKAJ-AJET A.Ş.</v>
@@ -4604,16 +4604,16 @@
     </row>
     <row r="183">
       <c r="A183" t="str">
-        <v>SYNPC000036</v>
+        <v>0GJG35T</v>
       </c>
       <c r="B183" t="str">
-        <v>Kullanıcı 256</v>
+        <v>Serkan Kaya</v>
       </c>
       <c r="C183" t="str">
         <v>SAHA OFISI-2</v>
       </c>
       <c r="D183" t="str">
-        <v>Sentetik OptiPlex SYN</v>
+        <v>Lenovo ThinkCentre M90</v>
       </c>
       <c r="E183" t="str">
         <v>TKAJ-AJET A.Ş.</v>
@@ -4627,16 +4627,16 @@
     </row>
     <row r="184">
       <c r="A184" t="str">
-        <v>SYNMN000057</v>
+        <v>CN001RS5C</v>
       </c>
       <c r="B184" t="str">
-        <v>Kullanıcı 239</v>
+        <v>Sultan Kara</v>
       </c>
       <c r="C184" t="str">
         <v>MERKEZ BINA</v>
       </c>
       <c r="D184" t="str">
-        <v>Sentetik Monitör Model</v>
+        <v>Dell U2419H</v>
       </c>
       <c r="E184" t="str">
         <v>TKAJ-AJET A.Ş.</v>
@@ -4650,16 +4650,16 @@
     </row>
     <row r="185">
       <c r="A185" t="str">
-        <v>SYNPC001868</v>
+        <v>PFAL079Z</v>
       </c>
       <c r="B185" t="str">
-        <v>Kullanıcı 302</v>
+        <v>Mustafa Şahin</v>
       </c>
       <c r="C185" t="str">
         <v>MERKEZ BINA</v>
       </c>
       <c r="D185" t="str">
-        <v>Sentetik ThinkPad SYN</v>
+        <v>Dell Latitude 5420</v>
       </c>
       <c r="E185" t="str">
         <v>TKAO-THY A.O.</v>
@@ -4673,16 +4673,16 @@
     </row>
     <row r="186">
       <c r="A186" t="str">
-        <v>SYNPC001416</v>
+        <v>0C2WN9V</v>
       </c>
       <c r="B186" t="str">
-        <v>Kullanıcı 263</v>
+        <v>Fatma Yıldız</v>
       </c>
       <c r="C186" t="str">
         <v>SAHA OFISI-2</v>
       </c>
       <c r="D186" t="str">
-        <v>Sentetik OptiPlex SYN</v>
+        <v>Lenovo ThinkCentre M90</v>
       </c>
       <c r="E186" t="str">
         <v>TKAO-THY A.O.</v>
@@ -4696,16 +4696,16 @@
     </row>
     <row r="187">
       <c r="A187" t="str">
-        <v>SYNPC000358</v>
+        <v>0JXCHNU</v>
       </c>
       <c r="B187" t="str">
-        <v>Kullanıcı 231</v>
+        <v>Tolga Yıldız</v>
       </c>
       <c r="C187" t="str">
         <v>SAHA OFISI-1</v>
       </c>
       <c r="D187" t="str">
-        <v>Sentetik OptiPlex SYN</v>
+        <v>Dell OptiPlex 5090</v>
       </c>
       <c r="E187" t="str">
         <v>TKAJ-AJET A.Ş.</v>
@@ -4719,16 +4719,16 @@
     </row>
     <row r="188">
       <c r="A188" t="str">
-        <v>SYNPC001397</v>
+        <v>0G46FTN</v>
       </c>
       <c r="B188" t="str">
-        <v>Kullanıcı 17</v>
+        <v>Fatma Doğan</v>
       </c>
       <c r="C188" t="str">
         <v>SAHA OFISI-2</v>
       </c>
       <c r="D188" t="str">
-        <v>Sentetik OptiPlex SYN</v>
+        <v>HP EliteDesk 800 G6</v>
       </c>
       <c r="E188" t="str">
         <v>TKAO-THY A.O.</v>

</xml_diff>